<commit_message>
exp typo test 09 30 results
</commit_message>
<xml_diff>
--- a/results/reliability_eval/reliability_eval_typo-test-09-30/Llama-3-8B_P17_char_insert_noise_typo3_sample_tok25_temp0.1_direct_completion_rep5_beams5_maxent20_rows100_raw_table_typo-test-09-30.xlsx
+++ b/results/reliability_eval/reliability_eval_typo-test-09-30/Llama-3-8B_P17_char_insert_noise_typo3_sample_tok25_temp0.1_direct_completion_rep5_beams5_maxent20_rows100_raw_table_typo-test-09-30.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>What is the location of Eibenstock?</t>
+          <t>What is= the locatio1n of Eiben0stock?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -509,33 +509,33 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>What is the location of Eibenstock? Answer: Eibenstock is located in the district of Zwickau in the Free State of Saxony in Germany. The town is</t>
+          <t>What is= the locatio1n of Eiben0stock? Answer: Eibenstock is located in the Ore Mountains in the German state of Saxony. The town is situated in the valley of</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Answer: Eibenstock is located in the district of Zwickau in the Free State of Saxony in Germany</t>
+          <t>Answer: Eibenstock is located in the Ore Mountains in the German state of Saxony. The town is situated in the valley of</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0.6514000296592712</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0.9830008745193481</v>
       </c>
       <c r="I2" t="n">
-        <v>-0</v>
+        <v>0.2792104780673981</v>
       </c>
       <c r="J2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>[(' E', 1.0), ('iben', 1.0), ('stock', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' district', 1.0), (' of', 1.0), (' Z', 1.0), ('wick', 1.0), ('au', 1.0), (' in', 1.0), (' the', 1.0), (' Free', 1.0), (' State', 1.0), (' of', 1.0), (' Sax', 1.0), ('ony', 1.0), (' in', 1.0), (' Germany', 1.0)]</t>
+          <t>[(' E', 1.0), ('iben', 1.0), ('stock', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Ore', 1.0), (' Mountains', 1.0), (' in', 1.0), (' the', 1.0), (' German', 1.0), (' state', 1.0), (' of', 1.0), (' Sax', 1.0), ('ony', 1.0), ('.', 1.0), (' The', 0.6514), (' town', 1.0), (' is', 1.0), (' situated', 1.0), (' in', 1.0), (' the', 1.0), (' valley', 1.0), (' of', 1.0)]</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -544,7 +544,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>What is the location of Eibenstock?</t>
+          <t>What is= the locatio1n of Eiben0stock?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -557,33 +557,33 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>What is the location of Eibenstock? Answer: Eibenstock is located in the district of Zwickau in the Free State of Saxony in Germany. The town is</t>
+          <t>What is= the locatio1n of Eiben0stock? Answer: Eibenstock is located in the Ore Mountains in the German state of Saxony. The town is situated in the valley of</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Answer: Eibenstock is located in the district of Zwickau in the Free State of Saxony in Germany</t>
+          <t>Answer: Eibenstock is located in the Ore Mountains in the German state of Saxony. The town is situated in the valley of</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0.6514000296592712</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0.9830008745193481</v>
       </c>
       <c r="I3" t="n">
-        <v>-0</v>
+        <v>0.2792104780673981</v>
       </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>[(' E', 1.0), ('iben', 1.0), ('stock', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' district', 1.0), (' of', 1.0), (' Z', 1.0), ('wick', 1.0), ('au', 1.0), (' in', 1.0), (' the', 1.0), (' Free', 1.0), (' State', 1.0), (' of', 1.0), (' Sax', 1.0), ('ony', 1.0), (' in', 1.0), (' Germany', 1.0)]</t>
+          <t>[(' E', 1.0), ('iben', 1.0), ('stock', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Ore', 1.0), (' Mountains', 1.0), (' in', 1.0), (' the', 1.0), (' German', 1.0), (' state', 1.0), (' of', 1.0), (' Sax', 1.0), ('ony', 1.0), ('.', 1.0), (' The', 0.6514), (' town', 1.0), (' is', 1.0), (' situated', 1.0), (' in', 1.0), (' the', 1.0), (' valley', 1.0), (' of', 1.0)]</t>
         </is>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -592,7 +592,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>What is the location of Eibenstock?</t>
+          <t>What is= the locatio1n of Eiben0stock?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -605,33 +605,33 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>What is the location of Eibenstock? Answer: Eibenstock is located in the district of Zwickau in the Free State of Saxony in Germany. The town is</t>
+          <t>What is= the locatio1n of Eiben0stock? Answer: Eibenstock is located in the Ore Mountains in the German state of Saxony. The town is situated in the valley of</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Answer: Eibenstock is located in the district of Zwickau in the Free State of Saxony in Germany</t>
+          <t>Answer: Eibenstock is located in the Ore Mountains in the German state of Saxony. The town is situated in the valley of</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0.6514000296592712</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>0.9830008745193481</v>
       </c>
       <c r="I4" t="n">
-        <v>-0</v>
+        <v>0.2792104780673981</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>[(' E', 1.0), ('iben', 1.0), ('stock', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' district', 1.0), (' of', 1.0), (' Z', 1.0), ('wick', 1.0), ('au', 1.0), (' in', 1.0), (' the', 1.0), (' Free', 1.0), (' State', 1.0), (' of', 1.0), (' Sax', 1.0), ('ony', 1.0), (' in', 1.0), (' Germany', 1.0)]</t>
+          <t>[(' E', 1.0), ('iben', 1.0), ('stock', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Ore', 1.0), (' Mountains', 1.0), (' in', 1.0), (' the', 1.0), (' German', 1.0), (' state', 1.0), (' of', 1.0), (' Sax', 1.0), ('ony', 1.0), ('.', 1.0), (' The', 0.6514), (' town', 1.0), (' is', 1.0), (' situated', 1.0), (' in', 1.0), (' the', 1.0), (' valley', 1.0), (' of', 1.0)]</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -640,7 +640,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>What is the location of Eibenstock?</t>
+          <t>What is= the locatio1n of Eiben0stock?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -653,33 +653,33 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>What is the location of Eibenstock? Answer: Eibenstock is located in the district of Zwickau in the Free State of Saxony in Germany. The town is</t>
+          <t>What is= the locatio1n of Eiben0stock? Answer: Eibenstock is located in the Ore Mountains in the German state of Saxony. It is a popular tourist destination known for</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Answer: Eibenstock is located in the district of Zwickau in the Free State of Saxony in Germany</t>
+          <t>Answer: Eibenstock is located in the Ore Mountains in the German state of Saxony. It is a popular tourist destination known for</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0.1743000000715256</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>0.9325065612792969</v>
       </c>
       <c r="I5" t="n">
-        <v>-0</v>
+        <v>0.7139387726783752</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>[(' E', 1.0), ('iben', 1.0), ('stock', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' district', 1.0), (' of', 1.0), (' Z', 1.0), ('wick', 1.0), ('au', 1.0), (' in', 1.0), (' the', 1.0), (' Free', 1.0), (' State', 1.0), (' of', 1.0), (' Sax', 1.0), ('ony', 1.0), (' in', 1.0), (' Germany', 1.0)]</t>
+          <t>[(' E', 1.0), ('iben', 1.0), ('stock', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Ore', 1.0), (' Mountains', 1.0), (' in', 1.0), (' the', 1.0), (' German', 1.0), (' state', 1.0), (' of', 1.0), (' Sax', 1.0), ('ony', 1.0), ('.', 1.0), (' It', 0.3486), (' is', 1.0), (' a', 0.5), (' popular', 1.0), (' tourist', 1.0), (' destination', 1.0), (' known', 1.0), (' for', 1.0)]</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -688,7 +688,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>What is the location of Eibenstock?</t>
+          <t>What is= the locatio1n of Eiben0stock?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -701,33 +701,33 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>What is the location of Eibenstock? Answer: Eibenstock is located in the district of Zwickau in the Free State of Saxony in Germany. The town is</t>
+          <t>What is= the locatio1n of Eiben0stock? Answer: Eibenstock is located in the Ore Mountains in the German state of Saxony. The town is situated in the valley of</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Answer: Eibenstock is located in the district of Zwickau in the Free State of Saxony in Germany</t>
+          <t>Answer: Eibenstock is located in the Ore Mountains in the German state of Saxony. The town is situated in the valley of</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0.6514000296592712</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>0.9830008745193481</v>
       </c>
       <c r="I6" t="n">
-        <v>-0</v>
+        <v>0.2792104780673981</v>
       </c>
       <c r="J6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>[(' E', 1.0), ('iben', 1.0), ('stock', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' district', 1.0), (' of', 1.0), (' Z', 1.0), ('wick', 1.0), ('au', 1.0), (' in', 1.0), (' the', 1.0), (' Free', 1.0), (' State', 1.0), (' of', 1.0), (' Sax', 1.0), ('ony', 1.0), (' in', 1.0), (' Germany', 1.0)]</t>
+          <t>[(' E', 1.0), ('iben', 1.0), ('stock', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Ore', 1.0), (' Mountains', 1.0), (' in', 1.0), (' the', 1.0), (' German', 1.0), (' state', 1.0), (' of', 1.0), (' Sax', 1.0), ('ony', 1.0), ('.', 1.0), (' The', 0.6514), (' town', 1.0), (' is', 1.0), (' situated', 1.0), (' in', 1.0), (' the', 1.0), (' valley', 1.0), (' of', 1.0)]</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -736,7 +736,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>What is the location of Simcoe Composite School?</t>
+          <t>What is t$he location `of Simc+oe Composite School?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -749,29 +749,29 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>What is the location of Simcoe Composite School? Answer: Simcoe Composite School is located in Simcoe, Ontario. What is the phone number of Simcoe Composite School? Answer:</t>
+          <t>What is t$he location `of Simc+oe Composite School? Answer: Simcoe Composite School is located at Simcoe ON N3Y 4K3. 2020-2021 School</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Answer: Simcoe Composite School is located in Simcoe, Ontario. What is the phone number of Simcoe Composite School? Answer:</t>
+          <t>Answer: Simcoe Composite School is located at Simcoe ON N3Y 4K3. 2020-2021 School</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>0.9460576772689819</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6931471824645996</v>
+        <v>-0</v>
       </c>
       <c r="J7" t="b">
         <v>0</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>[(' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), (' is', 1.0), (' located', 1.0), (' in', 0.5), (' Sim', 1.0), ('coe', 1.0), (',', 1.0), (' Ontario', 1.0), ('.', 1.0), (' What', 0.5), (' is', 1.0), (' the', 1.0), (' phone', 1.0), (' number', 1.0), (' of', 1.0), (' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), ('?', 1.0), (' Answer', 1.0), (':', 1.0)]</t>
+          <t>[(' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), (' is', 1.0), (' located', 1.0), (' at', 1.0), (' Sim', 1.0), ('coe', 1.0), (' ON', 1.0), (' N', 1.0), ('3', 1.0), ('Y', 1.0), (' ', 1.0), ('4', 1.0), ('K', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('202', 1.0), ('0', 1.0), ('-', 1.0), ('202', 1.0), ('1', 1.0), (' School', 1.0)]</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -784,7 +784,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>What is the location of Simcoe Composite School?</t>
+          <t>What is t$he location `of Simc+oe Composite School?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -797,29 +797,29 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>What is the location of Simcoe Composite School? Answer: Simcoe Composite School is located in Simcoe, Ontario. The school is located at 1 Parkhill Road West, Sim</t>
+          <t>What is t$he location `of Simc+oe Composite School? Answer: Simcoe Composite School is located at Simcoe ON N3Y 4K3. 2020-2021 School</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Answer: Simcoe Composite School is located in Simcoe, Ontario. The school is located at 1 Parkhill Road West, Sim</t>
+          <t>Answer: Simcoe Composite School is located at Simcoe ON N3Y 4K3. 2020-2021 School</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0.125</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>0.9201876521110535</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>1.039720773696899</v>
+        <v>-0</v>
       </c>
       <c r="J8" t="b">
         <v>0</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>[(' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), (' is', 1.0), (' located', 1.0), (' in', 0.5), (' Sim', 1.0), ('coe', 1.0), (',', 1.0), (' Ontario', 1.0), ('.', 1.0), (' The', 0.5), (' school', 1.0), (' is', 1.0), (' located', 1.0), (' at', 1.0), (' ', 1.0), ('1', 1.0), (' Park', 1.0), ('hill', 0.5), (' Road', 1.0), (' West', 1.0), (',', 1.0), (' Sim', 1.0)]</t>
+          <t>[(' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), (' is', 1.0), (' located', 1.0), (' at', 1.0), (' Sim', 1.0), ('coe', 1.0), (' ON', 1.0), (' N', 1.0), ('3', 1.0), ('Y', 1.0), (' ', 1.0), ('4', 1.0), ('K', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('202', 1.0), ('0', 1.0), ('-', 1.0), ('202', 1.0), ('1', 1.0), (' School', 1.0)]</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -832,7 +832,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>What is the location of Simcoe Composite School?</t>
+          <t>What is t$he location `of Simc+oe Composite School?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -845,29 +845,29 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>What is the location of Simcoe Composite School? Answer: Simcoe Composite School is located at 1 Simcoe Street, Simcoe, Ontario N3Y 4H3.</t>
+          <t>What is t$he location `of Simc+oe Composite School? Answer: Simcoe Composite School is located at Simcoe ON N3Y 4K3. 2020-2021 School</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Answer: Simcoe Composite School is located at 1 Simcoe Street, Simcoe, Ontario N3Y 4H3.</t>
+          <t>Answer: Simcoe Composite School is located at Simcoe ON N3Y 4K3. 2020-2021 School</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.09716250747442245</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>0.9109613299369812</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>1.23554515838623</v>
+        <v>-0</v>
       </c>
       <c r="J9" t="b">
         <v>0</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>[(' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), (' is', 1.0), (' located', 1.0), (' at', 0.5), (' ', 1.0), ('1', 1.0), (' Sim', 0.7773), ('coe', 1.0), (' Street', 1.0), (',', 1.0), (' Sim', 1.0), ('coe', 1.0), (',', 1.0), (' Ontario', 1.0), (' N', 0.5), ('3', 1.0), ('Y', 1.0), (' ', 1.0), ('4', 1.0), ('H', 1.0), ('3', 1.0), ('.', 0.5)]</t>
+          <t>[(' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), (' is', 1.0), (' located', 1.0), (' at', 1.0), (' Sim', 1.0), ('coe', 1.0), (' ON', 1.0), (' N', 1.0), ('3', 1.0), ('Y', 1.0), (' ', 1.0), ('4', 1.0), ('K', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('202', 1.0), ('0', 1.0), ('-', 1.0), ('202', 1.0), ('1', 1.0), (' School', 1.0)]</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -880,7 +880,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>What is the location of Simcoe Composite School?</t>
+          <t>What is t$he location `of Simc+oe Composite School?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -893,29 +893,29 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>What is the location of Simcoe Composite School? Answer: Simcoe Composite School is located in Simcoe, Ontario. What is the phone number of Simcoe Composite School? Answer:</t>
+          <t>What is t$he location `of Simc+oe Composite School? Answer: Simcoe Composite School is located at Simcoe ON N3Y 4K3. 2020-2021 School</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Answer: Simcoe Composite School is located in Simcoe, Ontario. What is the phone number of Simcoe Composite School? Answer:</t>
+          <t>Answer: Simcoe Composite School is located at Simcoe ON N3Y 4K3. 2020-2021 School</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>0.9460576772689819</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6931471824645996</v>
+        <v>-0</v>
       </c>
       <c r="J10" t="b">
         <v>0</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>[(' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), (' is', 1.0), (' located', 1.0), (' in', 0.5), (' Sim', 1.0), ('coe', 1.0), (',', 1.0), (' Ontario', 1.0), ('.', 1.0), (' What', 0.5), (' is', 1.0), (' the', 1.0), (' phone', 1.0), (' number', 1.0), (' of', 1.0), (' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), ('?', 1.0), (' Answer', 1.0), (':', 1.0)]</t>
+          <t>[(' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), (' is', 1.0), (' located', 1.0), (' at', 1.0), (' Sim', 1.0), ('coe', 1.0), (' ON', 1.0), (' N', 1.0), ('3', 1.0), ('Y', 1.0), (' ', 1.0), ('4', 1.0), ('K', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('202', 1.0), ('0', 1.0), ('-', 1.0), ('202', 1.0), ('1', 1.0), (' School', 1.0)]</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -928,7 +928,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>What is the location of Simcoe Composite School?</t>
+          <t>What is t$he location `of Simc+oe Composite School?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -941,31 +941,29 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the location of Simcoe Composite School? Answer: Simcoe Composite School is located at 1 Simcoe Street, Simcoe, Ontario N3Y 4H3.
-</t>
+          <t>What is t$he location `of Simc+oe Composite School? Answer: Simcoe Composite School is located at Simcoe ON N3Y 4K3. 2020-2021 School</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Answer: Simcoe Composite School is located at 1 Simcoe Street, Simcoe, Ontario N3Y 4H3.
-</t>
+          <t>Answer: Simcoe Composite School is located at Simcoe ON N3Y 4K3. 2020-2021 School</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0.09716250747442245</v>
+        <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>0.9109613299369812</v>
+        <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>1.23554515838623</v>
+        <v>-0</v>
       </c>
       <c r="J11" t="b">
         <v>0</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>[(' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), (' is', 1.0), (' located', 1.0), (' at', 0.5), (' ', 1.0), ('1', 1.0), (' Sim', 0.7773), ('coe', 1.0), (' Street', 1.0), (',', 1.0), (' Sim', 1.0), ('coe', 1.0), (',', 1.0), (' Ontario', 1.0), (' N', 0.5), ('3', 1.0), ('Y', 1.0), (' ', 1.0), ('4', 1.0), ('H', 1.0), ('3', 1.0), ('.\n', 0.5)]</t>
+          <t>[(' Sim', 1.0), ('coe', 1.0), (' Composite', 1.0), (' School', 1.0), (' is', 1.0), (' located', 1.0), (' at', 1.0), (' Sim', 1.0), ('coe', 1.0), (' ON', 1.0), (' N', 1.0), ('3', 1.0), ('Y', 1.0), (' ', 1.0), ('4', 1.0), ('K', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('202', 1.0), ('0', 1.0), ('-', 1.0), ('202', 1.0), ('1', 1.0), (' School', 1.0)]</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -978,7 +976,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>What is the location of Vrienden van het Platteland?</t>
+          <t>What is the loca9tion of' Vrienden~ van het Platteland?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -991,29 +989,29 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>What is the location of Vrienden van het Platteland? Answer: Vrienden van het Platteland is located in the province of Overijssel, the Netherlands. The coordinates of Vriend</t>
+          <t>What is the loca9tion of' Vrienden~ van het Platteland? Answer: Vrienden van het Platteland is located in the Netherlands.://www.://www. is the</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Answer: Vrienden van het Platteland is located in the province of Overijssel, the Netherlands</t>
+          <t>Answer: Vrienden van het Platteland is located in the Netherlands</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.7773000001907349</v>
+        <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>0.986828088760376</v>
+        <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>0.1958243548870087</v>
+        <v>-0</v>
       </c>
       <c r="J12" t="b">
         <v>1</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>[(' V', 1.0), ('riend', 1.0), ('en', 1.0), (' van', 1.0), (' het', 1.0), (' Platt', 1.0), ('eland', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' province', 1.0), (' of', 1.0), (' Over', 0.7773), ('ij', 1.0), ('ssel', 1.0), (',', 1.0), (' the', 1.0), (' Netherlands', 1.0)]</t>
+          <t>[(' V', 1.0), ('riend', 1.0), ('en', 1.0), (' van', 1.0), (' het', 1.0), (' Platt', 1.0), ('eland', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Netherlands', 1.0)]</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1026,7 +1024,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>What is the location of Vrienden van het Platteland?</t>
+          <t>What is the loca9tion of' Vrienden~ van het Platteland?</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1039,29 +1037,29 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>What is the location of Vrienden van het Platteland? Answer: Vrienden van het Platteland is located in the province of Overijssel, the Netherlands. The coordinates of Vriend</t>
+          <t>What is the loca9tion of' Vrienden~ van het Platteland? Answer: Vrienden van het Platteland is located in the Netherlands.://www.://www. is the</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Answer: Vrienden van het Platteland is located in the province of Overijssel, the Netherlands</t>
+          <t>Answer: Vrienden van het Platteland is located in the Netherlands</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0.7773000001907349</v>
+        <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>0.986828088760376</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>0.1958243548870087</v>
+        <v>-0</v>
       </c>
       <c r="J13" t="b">
         <v>1</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>[(' V', 1.0), ('riend', 1.0), ('en', 1.0), (' van', 1.0), (' het', 1.0), (' Platt', 1.0), ('eland', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' province', 1.0), (' of', 1.0), (' Over', 0.7773), ('ij', 1.0), ('ssel', 1.0), (',', 1.0), (' the', 1.0), (' Netherlands', 1.0)]</t>
+          <t>[(' V', 1.0), ('riend', 1.0), ('en', 1.0), (' van', 1.0), (' het', 1.0), (' Platt', 1.0), ('eland', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Netherlands', 1.0)]</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1074,7 +1072,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>What is the location of Vrienden van het Platteland?</t>
+          <t>What is the loca9tion of' Vrienden~ van het Platteland?</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1087,29 +1085,29 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>What is the location of Vrienden van het Platteland? Answer: Vrienden van het Platteland is located in the province of Overijssel, the Netherlands. The coordinates of Vriend</t>
+          <t>What is the loca9tion of' Vrienden~ van het Platteland? Answer: Vrienden van het Platteland is located in the Netherlands.://www.google.com/url?q=https://www.google</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Answer: Vrienden van het Platteland is located in the province of Overijssel, the Netherlands</t>
+          <t>Answer: Vrienden van het Platteland is located in the Netherlands</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0.7773000001907349</v>
+        <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>0.986828088760376</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>0.1958243548870087</v>
+        <v>-0</v>
       </c>
       <c r="J14" t="b">
         <v>1</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>[(' V', 1.0), ('riend', 1.0), ('en', 1.0), (' van', 1.0), (' het', 1.0), (' Platt', 1.0), ('eland', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' province', 1.0), (' of', 1.0), (' Over', 0.7773), ('ij', 1.0), ('ssel', 1.0), (',', 1.0), (' the', 1.0), (' Netherlands', 1.0)]</t>
+          <t>[(' V', 1.0), ('riend', 1.0), ('en', 1.0), (' van', 1.0), (' het', 1.0), (' Platt', 1.0), ('eland', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Netherlands', 1.0)]</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1122,7 +1120,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>What is the location of Vrienden van het Platteland?</t>
+          <t>What is the loca9tion of' Vrienden~ van het Platteland?</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1135,29 +1133,29 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>What is the location of Vrienden van het Platteland? Answer: Vrienden van het Platteland is located in the province of Limburg in the Netherlands. The coordinates of Vrienden</t>
+          <t>What is the loca9tion of' Vrienden~ van het Platteland? Answer: Vrienden van het Platteland is located in the Netherlands.://www.google.com/url?q=https://www.google</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Answer: Vrienden van het Platteland is located in the province of Limburg in the Netherlands</t>
+          <t>Answer: Vrienden van het Platteland is located in the Netherlands</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0.2226999849081039</v>
+        <v>1</v>
       </c>
       <c r="H15" t="n">
-        <v>0.9199457764625549</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>0.3344797492027283</v>
+        <v>-0</v>
       </c>
       <c r="J15" t="b">
         <v>1</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>[(' V', 1.0), ('riend', 1.0), ('en', 1.0), (' van', 1.0), (' het', 1.0), (' Platt', 1.0), ('eland', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' province', 1.0), (' of', 1.0), (' Lim', 0.2227), ('burg', 1.0), (' in', 1.0), (' the', 1.0), (' Netherlands', 1.0)]</t>
+          <t>[(' V', 1.0), ('riend', 1.0), ('en', 1.0), (' van', 1.0), (' het', 1.0), (' Platt', 1.0), ('eland', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Netherlands', 1.0)]</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1170,7 +1168,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>What is the location of Vrienden van het Platteland?</t>
+          <t>What is the loca9tion of' Vrienden~ van het Platteland?</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1183,29 +1181,29 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>What is the location of Vrienden van het Platteland? Answer: Vrienden van het Platteland is located in the province of Limburg in the Netherlands. The coordinates of Vrienden</t>
+          <t>What is the loca9tion of' Vrienden~ van het Platteland? Answer: Vrienden van het Platteland is located in the Netherlands.://www.google.com/url?q=https://www.google</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Answer: Vrienden van het Platteland is located in the province of Limburg in the Netherlands</t>
+          <t>Answer: Vrienden van het Platteland is located in the Netherlands</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>0.2226999849081039</v>
+        <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>0.9199457764625549</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>0.3344797492027283</v>
+        <v>-0</v>
       </c>
       <c r="J16" t="b">
         <v>1</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>[(' V', 1.0), ('riend', 1.0), ('en', 1.0), (' van', 1.0), (' het', 1.0), (' Platt', 1.0), ('eland', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' province', 1.0), (' of', 1.0), (' Lim', 0.2227), ('burg', 1.0), (' in', 1.0), (' the', 1.0), (' Netherlands', 1.0)]</t>
+          <t>[(' V', 1.0), ('riend', 1.0), ('en', 1.0), (' van', 1.0), (' het', 1.0), (' Platt', 1.0), ('eland', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Netherlands', 1.0)]</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1218,7 +1216,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>What is the location of Cunter?</t>
+          <t>What is th9e locatio&amp;n of Cunt_er?</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1231,33 +1229,33 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>What is the location of Cunter? Answer: Cunter is located in the state of Switzerland (Kanton Graubünden), in the district of Churwalden.</t>
+          <t>What is th9e locatio&amp;n of Cunt_er? Answer: The location of cunt_er is in the middle of the earth. It is a place where people go to have sex. It</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Answer: Cunter is located in the state of Switzerland (Kanton Graubünden)</t>
+          <t>Answer: The location of cunt_er is in the middle of the earth. It is a place where people go to have sex. It</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>0.5</v>
+        <v>0.1628500074148178</v>
       </c>
       <c r="H17" t="n">
-        <v>0.9258747100830078</v>
+        <v>0.9299755096435547</v>
       </c>
       <c r="I17" t="n">
-        <v>0.3465735912322998</v>
+        <v>0.9723576307296753</v>
       </c>
       <c r="J17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>[(' C', 1.0), ('unter', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' state', 0.5), (' of', 1.0), (' Switzerland', 1.0)]</t>
+          <t>[(' The', 0.6514), (' location', 1.0), (' of', 1.0), (' cunt', 1.0), ('_er', 1.0), (' is', 1.0), (' in', 1.0), (' the', 1.0), (' middle', 1.0), (' of', 1.0), (' the', 1.0), (' earth', 0.5), ('.', 1.0), (' It', 1.0), (' is', 1.0), (' a', 0.5), (' place', 1.0), (' where', 1.0), (' people', 1.0), (' go', 1.0), (' to', 1.0), (' have', 1.0), (' sex', 1.0), ('.', 1.0), (' It', 1.0)]</t>
         </is>
       </c>
       <c r="L17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1266,7 +1264,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>What is the location of Cunter?</t>
+          <t>What is th9e locatio&amp;n of Cunt_er?</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1279,33 +1277,33 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>What is the location of Cunter? Answer: Cunter is located in the state of Switzerland (Kanton Graubünden), in the district of Churwalden.</t>
+          <t>What is th9e locatio&amp;n of Cunt_er? Answer: The location of cunt_er is in the middle of the body. It is located between the legs and the anus. It is</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Answer: Cunter is located in the state of Switzerland (Kanton Graubünden)</t>
+          <t>Answer: The location of cunt_er is in the middle of the body. It is located between the legs and the anus. It is</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0.5</v>
+        <v>0.1628500074148178</v>
       </c>
       <c r="H18" t="n">
-        <v>0.9258747100830078</v>
+        <v>0.9299755096435547</v>
       </c>
       <c r="I18" t="n">
-        <v>0.3465735912322998</v>
+        <v>0.9723576307296753</v>
       </c>
       <c r="J18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>[(' C', 1.0), ('unter', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' state', 0.5), (' of', 1.0), (' Switzerland', 1.0)]</t>
+          <t>[(' The', 0.6514), (' location', 1.0), (' of', 1.0), (' cunt', 1.0), ('_er', 1.0), (' is', 1.0), (' in', 1.0), (' the', 1.0), (' middle', 1.0), (' of', 1.0), (' the', 1.0), (' body', 0.5), ('.', 1.0), (' It', 1.0), (' is', 1.0), (' located', 1.0), (' between', 1.0), (' the', 1.0), (' legs', 1.0), (' and', 1.0), (' the', 1.0), (' anus', 1.0), ('.', 1.0), (' It', 0.5), (' is', 1.0)]</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1314,7 +1312,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>What is the location of Cunter?</t>
+          <t>What is th9e locatio&amp;n of Cunt_er?</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1327,33 +1325,33 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>What is the location of Cunter? Answer: Cunter is located in the state of Switzerland (Kanton Graubünden), in the district of Churwalden.</t>
+          <t>What is th9e locatio&amp;n of Cunt_er? Answer: The location of cunt_er is in the middle of the body. It is located between the legs and the anus. The cunt</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Answer: Cunter is located in the state of Switzerland (Kanton Graubünden)</t>
+          <t>Answer: The location of cunt_er is in the middle of the body. It is located between the legs and the anus. The cunt</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>0.5</v>
+        <v>0.05676951259374619</v>
       </c>
       <c r="H19" t="n">
-        <v>0.9258747100830078</v>
+        <v>0.8915888071060181</v>
       </c>
       <c r="I19" t="n">
-        <v>0.3465735912322998</v>
+        <v>1.339722871780396</v>
       </c>
       <c r="J19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>[(' C', 1.0), ('unter', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' state', 0.5), (' of', 1.0), (' Switzerland', 1.0)]</t>
+          <t>[(' The', 0.6514), (' location', 1.0), (' of', 1.0), (' cunt', 1.0), ('_er', 1.0), (' is', 1.0), (' in', 1.0), (' the', 1.0), (' middle', 1.0), (' of', 1.0), (' the', 1.0), (' body', 0.5), ('.', 1.0), (' It', 1.0), (' is', 1.0), (' located', 1.0), (' between', 1.0), (' the', 1.0), (' legs', 1.0), (' and', 1.0), (' the', 1.0), (' anus', 1.0), ('.', 1.0), (' The', 0.5), (' cunt', 0.3486)]</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1362,7 +1360,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>What is the location of Cunter?</t>
+          <t>What is th9e locatio&amp;n of Cunt_er?</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1375,33 +1373,33 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>What is the location of Cunter? Answer: Cunter is located in the country of Switzerland. The latitude of Cunter is 46.8, and the longitude is</t>
+          <t>What is th9e locatio&amp;n of Cunt_er? Answer: The location of cunt_er is in the middle of the earth. It is a place where people go to have sex. It</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Answer: Cunter is located in the country of Switzerland</t>
+          <t>Answer: The location of cunt_er is in the middle of the earth. It is a place where people go to have sex. It</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>0.5</v>
+        <v>0.1628500074148178</v>
       </c>
       <c r="H20" t="n">
-        <v>0.9258747100830078</v>
+        <v>0.9299755096435547</v>
       </c>
       <c r="I20" t="n">
-        <v>0.3465735912322998</v>
+        <v>0.9723576307296753</v>
       </c>
       <c r="J20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>[(' C', 1.0), ('unter', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' country', 0.5), (' of', 1.0), (' Switzerland', 1.0)]</t>
+          <t>[(' The', 0.6514), (' location', 1.0), (' of', 1.0), (' cunt', 1.0), ('_er', 1.0), (' is', 1.0), (' in', 1.0), (' the', 1.0), (' middle', 1.0), (' of', 1.0), (' the', 1.0), (' earth', 0.5), ('.', 1.0), (' It', 1.0), (' is', 1.0), (' a', 0.5), (' place', 1.0), (' where', 1.0), (' people', 1.0), (' go', 1.0), (' to', 1.0), (' have', 1.0), (' sex', 1.0), ('.', 1.0), (' It', 1.0)]</t>
         </is>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1410,7 +1408,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>What is the location of Cunter?</t>
+          <t>What is th9e locatio&amp;n of Cunt_er?</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1423,33 +1421,33 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>What is the location of Cunter? Answer: Cunter is located in the state of Switzerland (Kanton Graubünden), in the district of Churwalden.</t>
+          <t>What is th9e locatio&amp;n of Cunt_er? Answer: The location of cunt_er is in the middle of the earth. It is located in the center of the earth. It is</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Answer: Cunter is located in the state of Switzerland (Kanton Graubünden)</t>
+          <t>Answer: The location of cunt_er is in the middle of the earth. It is located in the center of the earth. It is</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>0.5</v>
+        <v>0.08142500370740891</v>
       </c>
       <c r="H21" t="n">
-        <v>0.9258747100830078</v>
+        <v>0.9045453071594238</v>
       </c>
       <c r="I21" t="n">
-        <v>0.3465735912322998</v>
+        <v>1.318931221961975</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>[(' C', 1.0), ('unter', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' state', 0.5), (' of', 1.0), (' Switzerland', 1.0)]</t>
+          <t>[(' The', 0.6514), (' location', 1.0), (' of', 1.0), (' cunt', 1.0), ('_er', 1.0), (' is', 1.0), (' in', 1.0), (' the', 1.0), (' middle', 1.0), (' of', 1.0), (' the', 1.0), (' earth', 0.5), ('.', 1.0), (' It', 1.0), (' is', 1.0), (' located', 0.5), (' in', 0.5), (' the', 1.0), (' center', 1.0), (' of', 1.0), (' the', 1.0), (' earth', 1.0), ('.', 1.0), (' It', 1.0), (' is', 1.0)]</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1458,7 +1456,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>What is the location of Glencree?</t>
+          <t>Wh|at is the locatio~n [of Glencree?</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1471,33 +1469,33 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>What is the location of Glencree? Answer: Glencree is located in the Wicklow Mountains, 25 km south of Dublin city centre. It is situated on the</t>
+          <t>Wh|at is the locatio~n [of Glencree? Answer: It is situated in the county of Wicklow, in the south of Ireland, about 20 miles from Dublin. It is</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Answer: Glencree is located in the Wicklow Mountains, 25 km south of Dublin city centre. It is situated on the</t>
+          <t>Answer: It is situated in the county of Wicklow, in the south of Ireland</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>0.01855647377669811</v>
+        <v>0.25</v>
       </c>
       <c r="H22" t="n">
-        <v>0.8525891900062561</v>
+        <v>0.9117224812507629</v>
       </c>
       <c r="I22" t="n">
-        <v>1.393827795982361</v>
+        <v>0.6931471824645996</v>
       </c>
       <c r="J22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>[(' Gl', 1.0), ('enc', 1.0), ('ree', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Wick', 1.0), ('low', 1.0), (' Mountains', 1.0), (',', 1.0), (' ', 1.0), ('25', 0.2227), (' km', 0.5), (' south', 1.0), (' of', 1.0), (' Dublin', 1.0), (' city', 0.3333), (' centre', 1.0), ('.', 1.0), (' It', 1.0), (' is', 1.0), (' situated', 0.5), (' on', 1.0), (' the', 1.0)]</t>
+          <t>[(' It', 1.0), (' is', 1.0), (' situated', 1.0), (' in', 1.0), (' the', 1.0), (' county', 1.0), (' of', 1.0), (' Wick', 1.0), ('low', 1.0), (',', 1.0), (' in', 0.5), (' the', 1.0), (' south', 1.0), (' of', 0.5), (' Ireland', 1.0)]</t>
         </is>
       </c>
       <c r="L22" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="23">
@@ -1506,7 +1504,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>What is the location of Glencree?</t>
+          <t>Wh|at is the locatio~n [of Glencree?</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1519,33 +1517,33 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>What is the location of Glencree? Answer: Glencree is located in the Wicklow Mountains, 20 miles south of Dublin. It is 1.5 miles</t>
+          <t>Wh|at is the locatio~n [of Glencree? Answer: It is situated in the county of Wicklow, about 20 miles from Dublin, and 3 miles from the town of</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Answer: Glencree is located in the Wicklow Mountains, 20 miles south of Dublin. It is 1.5 miles</t>
+          <t>Answer: It is situated in the county of Wicklow, about 20 miles from Dublin, and 3 miles from the town of</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>0.1943250000476837</v>
+        <v>0.25</v>
       </c>
       <c r="H23" t="n">
-        <v>0.9365719556808472</v>
+        <v>0.9460576772689819</v>
       </c>
       <c r="I23" t="n">
-        <v>0.8889715671539307</v>
+        <v>0.6931471824645996</v>
       </c>
       <c r="J23" t="b">
         <v>0</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>[(' Gl', 1.0), ('enc', 1.0), ('ree', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Wick', 1.0), ('low', 1.0), (' Mountains', 1.0), (',', 1.0), (' ', 1.0), ('20', 0.7773), (' miles', 1.0), (' south', 1.0), (' of', 1.0), (' Dublin', 1.0), ('.', 0.5), (' It', 1.0), (' is', 1.0), (' ', 1.0), ('1', 0.5), ('.', 1.0), ('5', 1.0), (' miles', 1.0)]</t>
+          <t>[(' It', 1.0), (' is', 1.0), (' situated', 1.0), (' in', 1.0), (' the', 1.0), (' county', 1.0), (' of', 1.0), (' Wick', 1.0), ('low', 1.0), (',', 1.0), (' about', 0.5), (' ', 1.0), ('20', 1.0), (' miles', 1.0), (' from', 1.0), (' Dublin', 1.0), (',', 1.0), (' and', 1.0), (' ', 1.0), ('3', 0.5), (' miles', 1.0), (' from', 1.0), (' the', 1.0), (' town', 1.0), (' of', 1.0)]</t>
         </is>
       </c>
       <c r="L23" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="24">
@@ -1554,7 +1552,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>What is the location of Glencree?</t>
+          <t>Wh|at is the locatio~n [of Glencree?</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1567,33 +1565,33 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>What is the location of Glencree? Answer: Glencree is located in the Wicklow Mountains, 20 miles south of Dublin, Ireland. It is situated on the</t>
+          <t>Wh|at is the locatio~n [of Glencree? Answer: It is situated in the county of Wicklow, about 20 miles from Dublin, and 3 miles from the town of</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Answer: Glencree is located in the Wicklow Mountains, 20 miles south of Dublin, Ireland</t>
+          <t>Answer: It is situated in the county of Wicklow, about 20 miles from Dublin, and 3 miles from the town of</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>0.3886500000953674</v>
+        <v>0.25</v>
       </c>
       <c r="H24" t="n">
-        <v>0.951475977897644</v>
+        <v>0.9460576772689819</v>
       </c>
       <c r="I24" t="n">
-        <v>0.5423979759216309</v>
+        <v>0.6931471824645996</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>[(' Gl', 1.0), ('enc', 1.0), ('ree', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Wick', 1.0), ('low', 1.0), (' Mountains', 1.0), (',', 1.0), (' ', 1.0), ('20', 0.7773), (' miles', 1.0), (' south', 1.0), (' of', 1.0), (' Dublin', 1.0), (',', 0.5), (' Ireland', 1.0)]</t>
+          <t>[(' It', 1.0), (' is', 1.0), (' situated', 1.0), (' in', 1.0), (' the', 1.0), (' county', 1.0), (' of', 1.0), (' Wick', 1.0), ('low', 1.0), (',', 1.0), (' about', 0.5), (' ', 1.0), ('20', 1.0), (' miles', 1.0), (' from', 1.0), (' Dublin', 1.0), (',', 1.0), (' and', 1.0), (' ', 1.0), ('3', 0.5), (' miles', 1.0), (' from', 1.0), (' the', 1.0), (' town', 1.0), (' of', 1.0)]</t>
         </is>
       </c>
       <c r="L24" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="25">
@@ -1602,7 +1600,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>What is the location of Glencree?</t>
+          <t>Wh|at is the locatio~n [of Glencree?</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1615,33 +1613,33 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>What is the location of Glencree? Answer: Glencree is located in the Wicklow Mountains, 20 miles south of Dublin. It is 2 miles from the</t>
+          <t>Wh|at is the locatio~n [of Glencree? Answer: It is situated in the county of Wicklow, in the south of Ireland, about 20 miles from Dublin. It is</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Answer: Glencree is located in the Wicklow Mountains, 20 miles south of Dublin. It is 2 miles from the</t>
+          <t>Answer: It is situated in the county of Wicklow, in the south of Ireland</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>0.1943250000476837</v>
+        <v>0.25</v>
       </c>
       <c r="H25" t="n">
-        <v>0.9365719556808472</v>
+        <v>0.9117224812507629</v>
       </c>
       <c r="I25" t="n">
-        <v>0.8889715671539307</v>
+        <v>0.6931471824645996</v>
       </c>
       <c r="J25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>[(' Gl', 1.0), ('enc', 1.0), ('ree', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Wick', 1.0), ('low', 1.0), (' Mountains', 1.0), (',', 1.0), (' ', 1.0), ('20', 0.7773), (' miles', 1.0), (' south', 1.0), (' of', 1.0), (' Dublin', 1.0), ('.', 0.5), (' It', 1.0), (' is', 1.0), (' ', 1.0), ('2', 0.5), (' miles', 1.0), (' from', 1.0), (' the', 1.0)]</t>
+          <t>[(' It', 1.0), (' is', 1.0), (' situated', 1.0), (' in', 1.0), (' the', 1.0), (' county', 1.0), (' of', 1.0), (' Wick', 1.0), ('low', 1.0), (',', 1.0), (' in', 0.5), (' the', 1.0), (' south', 1.0), (' of', 0.5), (' Ireland', 1.0)]</t>
         </is>
       </c>
       <c r="L25" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="26">
@@ -1650,7 +1648,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>What is the location of Glencree?</t>
+          <t>Wh|at is the locatio~n [of Glencree?</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1663,33 +1661,33 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>What is the location of Glencree? Answer: Glencree is located in the Wicklow Mountains, 20 miles south of Dublin, Ireland. It is situated on the</t>
+          <t>Wh|at is the locatio~n [of Glencree? Answer: It is situated in the county of Wicklow, in the south-east of Ireland, about 20 miles from Dublin, and</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Answer: Glencree is located in the Wicklow Mountains, 20 miles south of Dublin, Ireland</t>
+          <t>Answer: It is situated in the county of Wicklow, in the south-east of Ireland</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>0.3886500000953674</v>
+        <v>0.25</v>
       </c>
       <c r="H26" t="n">
-        <v>0.951475977897644</v>
+        <v>0.9170040488243103</v>
       </c>
       <c r="I26" t="n">
-        <v>0.5423979759216309</v>
+        <v>0.6931471824645996</v>
       </c>
       <c r="J26" t="b">
         <v>1</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>[(' Gl', 1.0), ('enc', 1.0), ('ree', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' Wick', 1.0), ('low', 1.0), (' Mountains', 1.0), (',', 1.0), (' ', 1.0), ('20', 0.7773), (' miles', 1.0), (' south', 1.0), (' of', 1.0), (' Dublin', 1.0), (',', 0.5), (' Ireland', 1.0)]</t>
+          <t>[(' It', 1.0), (' is', 1.0), (' situated', 1.0), (' in', 1.0), (' the', 1.0), (' county', 1.0), (' of', 1.0), (' Wick', 1.0), ('low', 1.0), (',', 1.0), (' in', 0.5), (' the', 1.0), (' south', 1.0), ('-east', 0.5), (' of', 1.0), (' Ireland', 1.0)]</t>
         </is>
       </c>
       <c r="L26" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="27">
@@ -1698,7 +1696,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>What is the location of L'Escala?</t>
+          <t>W$hat is the locat?ion of L'Escal2a?</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1711,33 +1709,33 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>What is the location of L'Escala? Answer: L'Escala is located in the province of Girona, in the region of Catalonia, in the north-east of Spain</t>
+          <t xml:space="preserve">W$hat is the locat?ion of L'Escal2a? Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Answer: L'Escala is located in the province of Girona, in the region of Catalonia, in the north-east of Spain</t>
+          <t xml:space="preserve">Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H27" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>[(' L', 1.0), ("'E", 1.0), ('scala', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 0.5), (' province', 1.0), (' of', 1.0), (' G', 1.0), ('iron', 1.0), ('a', 1.0), (',', 1.0), (' in', 1.0), (' the', 1.0), (' region', 1.0), (' of', 1.0), (' Catalonia', 1.0), (',', 1.0), (' in', 1.0), (' the', 1.0), (' north', 1.0), ('-east', 1.0), (' of', 1.0), (' Spain', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' ', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('4', 1.0), ('.', 1.0), (' ', 1.0), ('5', 1.0), ('.', 1.0), (' ', 1.0), ('6', 1.0), ('.', 1.0), (' ', 1.0), ('7', 1.0), ('.', 1.0), (' ', 1.0), ('8', 1.0), ('.', 1.0), (' ', 1.0)]</t>
         </is>
       </c>
       <c r="L27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1746,7 +1744,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>What is the location of L'Escala?</t>
+          <t>W$hat is the locat?ion of L'Escal2a?</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1759,33 +1757,33 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>What is the location of L'Escala? Answer: L'Escala is located in the province of Girona, in the region of Catalonia, in the north-east of Spain</t>
+          <t xml:space="preserve">W$hat is the locat?ion of L'Escal2a? Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Answer: L'Escala is located in the province of Girona, in the region of Catalonia, in the north-east of Spain</t>
+          <t xml:space="preserve">Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H28" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>[(' L', 1.0), ("'E", 1.0), ('scala', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 0.5), (' province', 1.0), (' of', 1.0), (' G', 1.0), ('iron', 1.0), ('a', 1.0), (',', 1.0), (' in', 1.0), (' the', 1.0), (' region', 1.0), (' of', 1.0), (' Catalonia', 1.0), (',', 1.0), (' in', 1.0), (' the', 1.0), (' north', 1.0), ('-east', 1.0), (' of', 1.0), (' Spain', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' ', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('4', 1.0), ('.', 1.0), (' ', 1.0), ('5', 1.0), ('.', 1.0), (' ', 1.0), ('6', 1.0), ('.', 1.0), (' ', 1.0), ('7', 1.0), ('.', 1.0), (' ', 1.0), ('8', 1.0), ('.', 1.0), (' ', 1.0)]</t>
         </is>
       </c>
       <c r="L28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1794,7 +1792,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>What is the location of L'Escala?</t>
+          <t>W$hat is the locat?ion of L'Escal2a?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1807,33 +1805,33 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>What is the location of L'Escala? Answer: L'Escala is located in the province of Girona, in the region of Catalonia, in the north-east of Spain</t>
+          <t xml:space="preserve">W$hat is the locat?ion of L'Escal2a? Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Answer: L'Escala is located in the province of Girona, in the region of Catalonia, in the north-east of Spain</t>
+          <t xml:space="preserve">Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H29" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>[(' L', 1.0), ("'E", 1.0), ('scala', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 0.5), (' province', 1.0), (' of', 1.0), (' G', 1.0), ('iron', 1.0), ('a', 1.0), (',', 1.0), (' in', 1.0), (' the', 1.0), (' region', 1.0), (' of', 1.0), (' Catalonia', 1.0), (',', 1.0), (' in', 1.0), (' the', 1.0), (' north', 1.0), ('-east', 1.0), (' of', 1.0), (' Spain', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' ', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('4', 1.0), ('.', 1.0), (' ', 1.0), ('5', 1.0), ('.', 1.0), (' ', 1.0), ('6', 1.0), ('.', 1.0), (' ', 1.0), ('7', 1.0), ('.', 1.0), (' ', 1.0), ('8', 1.0), ('.', 1.0), (' ', 1.0)]</t>
         </is>
       </c>
       <c r="L29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1842,7 +1840,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>What is the location of L'Escala?</t>
+          <t>W$hat is the locat?ion of L'Escal2a?</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1855,33 +1853,33 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>What is the location of L'Escala? Answer: L'Escala is located in the province of Girona, in the region of Catalonia, in the north-east of Spain</t>
+          <t xml:space="preserve">W$hat is the locat?ion of L'Escal2a? Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Answer: L'Escala is located in the province of Girona, in the region of Catalonia, in the north-east of Spain</t>
+          <t xml:space="preserve">Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>[(' L', 1.0), ("'E", 1.0), ('scala', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 0.5), (' province', 1.0), (' of', 1.0), (' G', 1.0), ('iron', 1.0), ('a', 1.0), (',', 1.0), (' in', 1.0), (' the', 1.0), (' region', 1.0), (' of', 1.0), (' Catalonia', 1.0), (',', 1.0), (' in', 1.0), (' the', 1.0), (' north', 1.0), ('-east', 1.0), (' of', 1.0), (' Spain', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' ', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('4', 1.0), ('.', 1.0), (' ', 1.0), ('5', 1.0), ('.', 1.0), (' ', 1.0), ('6', 1.0), ('.', 1.0), (' ', 1.0), ('7', 1.0), ('.', 1.0), (' ', 1.0), ('8', 1.0), ('.', 1.0), (' ', 1.0)]</t>
         </is>
       </c>
       <c r="L30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1890,7 +1888,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>What is the location of L'Escala?</t>
+          <t>W$hat is the locat?ion of L'Escal2a?</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1903,33 +1901,33 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>What is the location of L'Escala? Answer: L'Escala is located in Spain (Catalonia) and time zone Europe/Madrid. Coordinates of L'Escala</t>
+          <t xml:space="preserve">W$hat is the locat?ion of L'Escal2a? Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Answer: L'Escala is located in Spain (Catalonia) and time zone Europe/Madrid</t>
+          <t xml:space="preserve">Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H31" t="n">
-        <v>0.9057236313819885</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>[(' L', 1.0), ("'E", 1.0), ('scala', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Spain', 0.5)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' ', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('4', 1.0), ('.', 1.0), (' ', 1.0), ('5', 1.0), ('.', 1.0), (' ', 1.0), ('6', 1.0), ('.', 1.0), (' ', 1.0), ('7', 1.0), ('.', 1.0), (' ', 1.0), ('8', 1.0), ('.', 1.0), (' ', 1.0)]</t>
         </is>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -1938,7 +1936,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>What is the location of Wismar?</t>
+          <t>What{ is the locat4ion of Wism,ar?</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1951,29 +1949,29 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>What is the location of Wismar? Answer: Wismar is located in the north of Germany, in the state of Mecklenburg-Vorpommern. The</t>
+          <t>What{ is the locat4ion of Wism,ar? Answer: Wismar is located in Germany. It is the capital of the Mecklenburg-Vorpommern state. It</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Answer: Wismar is located in the north of Germany</t>
+          <t>Answer: Wismar is located in Germany</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H32" t="n">
-        <v>0.9330329895019531</v>
+        <v>1</v>
       </c>
       <c r="I32" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J32" t="b">
         <v>1</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>[(' W', 1.0), ('ism', 1.0), ('ar', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' north', 0.5), (' of', 1.0), (' Germany', 1.0)]</t>
+          <t>[(' W', 1.0), ('ism', 1.0), ('ar', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Germany', 1.0)]</t>
         </is>
       </c>
       <c r="L32" t="n">
@@ -1986,7 +1984,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>What is the location of Wismar?</t>
+          <t>What{ is the locat4ion of Wism,ar?</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1999,29 +1997,29 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>What is the location of Wismar? Answer: Wismar is located in the north of Germany, in the state of Mecklenburg-Vorpommern. The</t>
+          <t>What{ is the locat4ion of Wism,ar? Answer: Wismar is located in Germany. What is the population of Wismar? Answer: The population of Wismar</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Answer: Wismar is located in the north of Germany</t>
+          <t>Answer: Wismar is located in Germany</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H33" t="n">
-        <v>0.9330329895019531</v>
+        <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J33" t="b">
         <v>1</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>[(' W', 1.0), ('ism', 1.0), ('ar', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' north', 0.5), (' of', 1.0), (' Germany', 1.0)]</t>
+          <t>[(' W', 1.0), ('ism', 1.0), ('ar', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Germany', 1.0)]</t>
         </is>
       </c>
       <c r="L33" t="n">
@@ -2034,7 +2032,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>What is the location of Wismar?</t>
+          <t>What{ is the locat4ion of Wism,ar?</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2047,29 +2045,29 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>What is the location of Wismar? Answer: Wismar is located in the north of Germany, in the state of Mecklenburg-Vorpommern. The</t>
+          <t>What{ is the locat4ion of Wism,ar? Answer: Wismar is located in Germany. It is the capital of the Mecklenburg-Vorpommern region. It</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Answer: Wismar is located in the north of Germany</t>
+          <t>Answer: Wismar is located in Germany</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H34" t="n">
-        <v>0.9330329895019531</v>
+        <v>1</v>
       </c>
       <c r="I34" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J34" t="b">
         <v>1</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>[(' W', 1.0), ('ism', 1.0), ('ar', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' north', 0.5), (' of', 1.0), (' Germany', 1.0)]</t>
+          <t>[(' W', 1.0), ('ism', 1.0), ('ar', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Germany', 1.0)]</t>
         </is>
       </c>
       <c r="L34" t="n">
@@ -2082,7 +2080,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>What is the location of Wismar?</t>
+          <t>What{ is the locat4ion of Wism,ar?</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2095,29 +2093,29 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>What is the location of Wismar? Answer: Wismar is located in the north of Germany, in the state of Mecklenburg-Vorpommern. The</t>
+          <t>What{ is the locat4ion of Wism,ar? Answer: Wismar is located in Germany. It is the capital of the Mecklenburg-Vorpommern state. It</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Answer: Wismar is located in the north of Germany</t>
+          <t>Answer: Wismar is located in Germany</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H35" t="n">
-        <v>0.9330329895019531</v>
+        <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J35" t="b">
         <v>1</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>[(' W', 1.0), ('ism', 1.0), ('ar', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' north', 0.5), (' of', 1.0), (' Germany', 1.0)]</t>
+          <t>[(' W', 1.0), ('ism', 1.0), ('ar', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Germany', 1.0)]</t>
         </is>
       </c>
       <c r="L35" t="n">
@@ -2130,7 +2128,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>What is the location of Wismar?</t>
+          <t>What{ is the locat4ion of Wism,ar?</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2143,29 +2141,29 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>What is the location of Wismar? Answer: Wismar is located in the north of Germany, in the state of Mecklenburg-Vorpommern. The</t>
+          <t>What{ is the locat4ion of Wism,ar? Answer: Wismar is located in Germany. It is the capital of the Mecklenburg-Vorpommern region. It</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Answer: Wismar is located in the north of Germany</t>
+          <t>Answer: Wismar is located in Germany</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H36" t="n">
-        <v>0.9330329895019531</v>
+        <v>1</v>
       </c>
       <c r="I36" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J36" t="b">
         <v>1</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>[(' W', 1.0), ('ism', 1.0), ('ar', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' north', 0.5), (' of', 1.0), (' Germany', 1.0)]</t>
+          <t>[(' W', 1.0), ('ism', 1.0), ('ar', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Germany', 1.0)]</t>
         </is>
       </c>
       <c r="L36" t="n">
@@ -2178,7 +2176,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>What is the location of Namba Station?</t>
+          <t>Wh1at is the; location of Namba S0tation?</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2191,29 +2189,29 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>What is the location of Namba Station? Answer: Namba Station is located in Osaka, Japan. Namba Station is located in Osaka, Japan. Namba Station is located</t>
+          <t>Wh1at is the; location of Namba S0tation? Answer: Namba Station is located in the Namba district of Osaka, Japan. It is a major transportation hub for the city,</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Answer: Namba Station is located in Osaka, Japan</t>
+          <t>Answer: Namba Station is located in the Namba district of Osaka, Japan</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>0.5</v>
+        <v>0.3886500000953674</v>
       </c>
       <c r="H37" t="n">
-        <v>0.9258747100830078</v>
+        <v>0.9347226619720459</v>
       </c>
       <c r="I37" t="n">
-        <v>0.3465735912322998</v>
+        <v>0.5423979759216309</v>
       </c>
       <c r="J37" t="b">
         <v>1</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>[(' N', 1.0), ('amba', 1.0), (' Station', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Osaka', 0.5), (',', 1.0), (' Japan', 1.0)]</t>
+          <t>[(' N', 0.7773), ('amba', 1.0), (' Station', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' N', 1.0), ('amba', 1.0), (' district', 0.5), (' of', 1.0), (' Osaka', 1.0), (',', 1.0), (' Japan', 1.0)]</t>
         </is>
       </c>
       <c r="L37" t="n">
@@ -2226,7 +2224,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>What is the location of Namba Station?</t>
+          <t>Wh1at is the; location of Namba S0tation?</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2239,29 +2237,29 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>What is the location of Namba Station? Answer: Namba Station is located in Osaka, Japan. Namba Station is located in Osaka, Japan. Namba Station is located</t>
+          <t>Wh1at is the; location of Namba S0tation? Answer: Namba Station is located in the Namba district of Osaka, Japan. It is a major transportation hub for the city,</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Answer: Namba Station is located in Osaka, Japan</t>
+          <t>Answer: Namba Station is located in the Namba district of Osaka, Japan</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>0.5</v>
+        <v>0.3886500000953674</v>
       </c>
       <c r="H38" t="n">
-        <v>0.9258747100830078</v>
+        <v>0.9347226619720459</v>
       </c>
       <c r="I38" t="n">
-        <v>0.3465735912322998</v>
+        <v>0.5423979759216309</v>
       </c>
       <c r="J38" t="b">
         <v>1</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>[(' N', 1.0), ('amba', 1.0), (' Station', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Osaka', 0.5), (',', 1.0), (' Japan', 1.0)]</t>
+          <t>[(' N', 0.7773), ('amba', 1.0), (' Station', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' N', 1.0), ('amba', 1.0), (' district', 0.5), (' of', 1.0), (' Osaka', 1.0), (',', 1.0), (' Japan', 1.0)]</t>
         </is>
       </c>
       <c r="L38" t="n">
@@ -2274,7 +2272,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>What is the location of Namba Station?</t>
+          <t>Wh1at is the; location of Namba S0tation?</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2287,7 +2285,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>What is the location of Namba Station? Answer: Namba Station is located in the Namba district of Osaka, Japan. It is a major transportation hub in the city,</t>
+          <t>Wh1at is the; location of Namba S0tation? Answer: Namba Station is located in the Namba district of Osaka, Japan. It is a major transportation hub for the city,</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2296,20 +2294,20 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>0.5</v>
+        <v>0.3886500000953674</v>
       </c>
       <c r="H39" t="n">
-        <v>0.9516951441764832</v>
+        <v>0.9347226619720459</v>
       </c>
       <c r="I39" t="n">
-        <v>0.3465735912322998</v>
+        <v>0.5423979759216309</v>
       </c>
       <c r="J39" t="b">
         <v>1</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>[(' N', 1.0), ('amba', 1.0), (' Station', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 0.5), (' N', 1.0), ('amba', 1.0), (' district', 1.0), (' of', 1.0), (' Osaka', 1.0), (',', 1.0), (' Japan', 1.0)]</t>
+          <t>[(' N', 0.7773), ('amba', 1.0), (' Station', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' N', 1.0), ('amba', 1.0), (' district', 0.5), (' of', 1.0), (' Osaka', 1.0), (',', 1.0), (' Japan', 1.0)]</t>
         </is>
       </c>
       <c r="L39" t="n">
@@ -2322,7 +2320,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>What is the location of Namba Station?</t>
+          <t>Wh1at is the; location of Namba S0tation?</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2335,29 +2333,29 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>What is the location of Namba Station? Answer: Namba Station is located in Osaka, Japan. Namba Station is located in Osaka, Japan. Namba Station is located</t>
+          <t>Wh1at is the; location of Namba S0tation? Answer: Osaka, Japan. The Namba Station is a major railway station in Osaka, Japan. It is located in the Namba</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Answer: Namba Station is located in Osaka, Japan</t>
+          <t>Answer: Osaka, Japan</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>0.5</v>
+        <v>0.2226999849081039</v>
       </c>
       <c r="H40" t="n">
-        <v>0.9258747100830078</v>
+        <v>0.6061406135559082</v>
       </c>
       <c r="I40" t="n">
-        <v>0.3465735912322998</v>
+        <v>0.3344797492027283</v>
       </c>
       <c r="J40" t="b">
         <v>1</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>[(' N', 1.0), ('amba', 1.0), (' Station', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Osaka', 0.5), (',', 1.0), (' Japan', 1.0)]</t>
+          <t>[(' Osaka', 0.2227), (',', 1.0), (' Japan', 1.0)]</t>
         </is>
       </c>
       <c r="L40" t="n">
@@ -2370,7 +2368,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>What is the location of Namba Station?</t>
+          <t>Wh1at is the; location of Namba S0tation?</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2383,29 +2381,29 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>What is the location of Namba Station? Answer: Namba Station is located in Osaka, Japan. Namba Station is located in Osaka, Japan. Namba Station is located</t>
+          <t>Wh1at is the; location of Namba S0tation? Answer: Namba Station is located in the Namba district of Osaka, Japan. It is a major transportation hub in the city,</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Answer: Namba Station is located in Osaka, Japan</t>
+          <t>Answer: Namba Station is located in the Namba district of Osaka, Japan</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>0.5</v>
+        <v>0.3886500000953674</v>
       </c>
       <c r="H41" t="n">
-        <v>0.9258747100830078</v>
+        <v>0.9347226619720459</v>
       </c>
       <c r="I41" t="n">
-        <v>0.3465735912322998</v>
+        <v>0.5423979759216309</v>
       </c>
       <c r="J41" t="b">
         <v>1</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>[(' N', 1.0), ('amba', 1.0), (' Station', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Osaka', 0.5), (',', 1.0), (' Japan', 1.0)]</t>
+          <t>[(' N', 0.7773), ('amba', 1.0), (' Station', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' N', 1.0), ('amba', 1.0), (' district', 0.5), (' of', 1.0), (' Osaka', 1.0), (',', 1.0), (' Japan', 1.0)]</t>
         </is>
       </c>
       <c r="L41" t="n">
@@ -2418,7 +2416,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>What is the location of 2010 Belgian federal election?</t>
+          <t>W-hat [is the locat*ion of 2010 Belgian federal election?</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2431,9 +2429,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>What is the location of 2010 Belgian federal election? Answer: Belgium
-What is the location of 2010 Belgian federal election?
-Belgium is a country located in the Western Europe region</t>
+          <t>W-hat [is the locat*ion of 2010 Belgian federal election? Answer: Belgium. The election was held on 13 June 2010. The election was held on 13 June 2010</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2459,7 +2455,7 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="43">
@@ -2468,7 +2464,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>What is the location of 2010 Belgian federal election?</t>
+          <t>W-hat [is the locat*ion of 2010 Belgian federal election?</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2481,34 +2477,33 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>What is the location of 2010 Belgian federal election? Answer: 2010 Belgian federal election was held in Belgium. 2010 Belgian federal election was held in Belgium.
-What is the</t>
+          <t>W-hat [is the locat*ion of 2010 Belgian federal election? Answer: Belgium. The election was held on 13 June 2010. The election was held on 13 June 2010</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Answer: 2010 Belgian federal election was held in Belgium</t>
+          <t>Answer: Belgium</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>0.3486000001430511</v>
+        <v>0.6514000296592712</v>
       </c>
       <c r="H43" t="n">
-        <v>0.8999797701835632</v>
+        <v>0.6514000296592712</v>
       </c>
       <c r="I43" t="n">
-        <v>0.3673651814460754</v>
+        <v>0.2792104780673981</v>
       </c>
       <c r="J43" t="b">
         <v>1</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>[(' ', 0.3486), ('201', 1.0), ('0', 1.0), (' Belgian', 1.0), (' federal', 1.0), (' election', 1.0), (' was', 1.0), (' held', 1.0), (' in', 1.0), (' Belgium', 1.0)]</t>
+          <t>[(' Belgium', 0.6514)]</t>
         </is>
       </c>
       <c r="L43" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="44">
@@ -2517,7 +2512,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>What is the location of 2010 Belgian federal election?</t>
+          <t>W-hat [is the locat*ion of 2010 Belgian federal election?</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2530,35 +2525,35 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>What is the location of 2010 Belgian federal election? Answer: Belgium
-What is the location of 2010 Belgian federal election?
-Belgium is a country located in the Western Europe region</t>
+          <t>W-hat [is the locat*ion of 2010 Belgian federal election? Answer: 2010 Belgian federal election
+W-hat [is the locat*ion of 2010 Belgian federal election?</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Answer: Belgium</t>
+          <t>Answer: 2010 Belgian federal election
+W-hat [is the locat*ion of 2010 Belgian federal election?</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>0.6514000296592712</v>
+        <v>0.3486000001430511</v>
       </c>
       <c r="H44" t="n">
-        <v>0.6514000296592712</v>
+        <v>0.9587228894233704</v>
       </c>
       <c r="I44" t="n">
-        <v>0.2792104780673981</v>
+        <v>0.3673651814460754</v>
       </c>
       <c r="J44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>[(' Belgium', 0.6514)]</t>
+          <t>[(' ', 0.3486), ('201', 1.0), ('0', 1.0), (' Belgian', 1.0), (' federal', 1.0), (' election', 1.0), ('\n', 1.0), ('W', 1.0), ('-h', 1.0), ('at', 1.0), (' [', 1.0), ('is', 1.0), (' the', 1.0), (' loc', 1.0), ('at', 1.0), ('*', 1.0), ('ion', 1.0), (' of', 1.0), (' ', 1.0), ('201', 1.0), ('0', 1.0), (' Belgian', 1.0), (' federal', 1.0), (' election', 1.0), ('?', 1.0)]</t>
         </is>
       </c>
       <c r="L44" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="45">
@@ -2567,7 +2562,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>What is the location of 2010 Belgian federal election?</t>
+          <t>W-hat [is the locat*ion of 2010 Belgian federal election?</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2580,9 +2575,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>What is the location of 2010 Belgian federal election? Answer: Belgium
-What is the location of 2010 Belgian federal election?
-Belgium is a country located in Western Europe. It</t>
+          <t>W-hat [is the locat*ion of 2010 Belgian federal election? Answer: Belgium. The election was held on 13 June 2010. The Christian Democratic and Flemish (CD&amp;V)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2608,7 +2601,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="46">
@@ -2617,7 +2610,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>What is the location of 2010 Belgian federal election?</t>
+          <t>W-hat [is the locat*ion of 2010 Belgian federal election?</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2630,33 +2623,33 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>What is the location of 2010 Belgian federal election? Answer: 2010 Belgian federal election was held in Belgium.://en.wikipedia.org/wiki/2010_Belgian</t>
+          <t>W-hat [is the locat*ion of 2010 Belgian federal election? Answer: Belgium. The election was held on 13 June 2010. The Christian Democratic and Flemish (CD&amp;V)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Answer: 2010 Belgian federal election was held in Belgium</t>
+          <t>Answer: Belgium</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>0.3486000001430511</v>
+        <v>0.6514000296592712</v>
       </c>
       <c r="H46" t="n">
-        <v>0.8999797701835632</v>
+        <v>0.6514000296592712</v>
       </c>
       <c r="I46" t="n">
-        <v>0.3673651814460754</v>
+        <v>0.2792104780673981</v>
       </c>
       <c r="J46" t="b">
         <v>1</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>[(' ', 0.3486), ('201', 1.0), ('0', 1.0), (' Belgian', 1.0), (' federal', 1.0), (' election', 1.0), (' was', 1.0), (' held', 1.0), (' in', 1.0), (' Belgium', 1.0)]</t>
+          <t>[(' Belgium', 0.6514)]</t>
         </is>
       </c>
       <c r="L46" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="47">
@@ -2665,7 +2658,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>What is the location of CFMJ?</t>
+          <t>W6hat i"s the location% of CFMJ?</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2678,31 +2671,29 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>What is the location of CFMJ? Answer: CFMJ is located at 101 The East Mall, Toronto, Ontario, M9B 6K1.
-What is</t>
+          <t xml:space="preserve">W6hat i"s the location% of CFMJ? Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Answer: CFMJ is located at 101 The East Mall, Toronto, Ontario, M9B 6K1.
-What is</t>
+          <t xml:space="preserve">Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H47" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I47" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J47" t="b">
         <v>0</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>[(' CF', 1.0), ('MJ', 1.0), (' is', 1.0), (' located', 1.0), (' at', 1.0), (' ', 1.0), ('101', 0.5), (' The', 1.0), (' East', 1.0), (' Mall', 1.0), (',', 1.0), (' Toronto', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' M', 1.0), ('9', 1.0), ('B', 1.0), (' ', 1.0), ('6', 1.0), ('K', 1.0), ('1', 1.0), ('.\n', 1.0), ('What', 1.0), (' is', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' ', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('4', 1.0), ('.', 1.0), (' ', 1.0), ('5', 1.0), ('.', 1.0), (' ', 1.0), ('6', 1.0), ('.', 1.0), (' ', 1.0), ('7', 1.0), ('.', 1.0), (' ', 1.0), ('8', 1.0), ('.', 1.0), (' ', 1.0)]</t>
         </is>
       </c>
       <c r="L47" t="n">
@@ -2715,7 +2706,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>What is the location of CFMJ?</t>
+          <t>W6hat i"s the location% of CFMJ?</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2728,31 +2719,29 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>What is the location of CFMJ? Answer: CFMJ is located at 550 Bay Street, Toronto, Ontario, M5G 2M9.
-What is the</t>
+          <t xml:space="preserve">W6hat i"s the location% of CFMJ? Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Answer: CFMJ is located at 550 Bay Street, Toronto, Ontario, M5G 2M9.
-What is the</t>
+          <t xml:space="preserve">Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="H48" t="n">
-        <v>0.9460576772689819</v>
+        <v>1</v>
       </c>
       <c r="I48" t="n">
-        <v>0.6931471824645996</v>
+        <v>-0</v>
       </c>
       <c r="J48" t="b">
         <v>0</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>[(' CF', 1.0), ('MJ', 1.0), (' is', 1.0), (' located', 1.0), (' at', 1.0), (' ', 1.0), ('550', 0.5), (' Bay', 1.0), (' Street', 1.0), (',', 1.0), (' Toronto', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' M', 0.5), ('5', 1.0), ('G', 1.0), (' ', 1.0), ('2', 1.0), ('M', 1.0), ('9', 1.0), ('.\n', 1.0), ('What', 1.0), (' is', 1.0), (' the', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' ', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('4', 1.0), ('.', 1.0), (' ', 1.0), ('5', 1.0), ('.', 1.0), (' ', 1.0), ('6', 1.0), ('.', 1.0), (' ', 1.0), ('7', 1.0), ('.', 1.0), (' ', 1.0), ('8', 1.0), ('.', 1.0), (' ', 1.0)]</t>
         </is>
       </c>
       <c r="L48" t="n">
@@ -2765,7 +2754,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>What is the location of CFMJ?</t>
+          <t>W6hat i"s the location% of CFMJ?</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2778,31 +2767,29 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>What is the location of CFMJ? Answer: CFMJ is located at 101 The East Mall, Toronto, Ontario, M9B 6K1.
-What is</t>
+          <t xml:space="preserve">W6hat i"s the location% of CFMJ? Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Answer: CFMJ is located at 101 The East Mall, Toronto, Ontario, M9B 6K1.
-What is</t>
+          <t xml:space="preserve">Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H49" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J49" t="b">
         <v>0</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>[(' CF', 1.0), ('MJ', 1.0), (' is', 1.0), (' located', 1.0), (' at', 1.0), (' ', 1.0), ('101', 0.5), (' The', 1.0), (' East', 1.0), (' Mall', 1.0), (',', 1.0), (' Toronto', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' M', 1.0), ('9', 1.0), ('B', 1.0), (' ', 1.0), ('6', 1.0), ('K', 1.0), ('1', 1.0), ('.\n', 1.0), ('What', 1.0), (' is', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' ', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('4', 1.0), ('.', 1.0), (' ', 1.0), ('5', 1.0), ('.', 1.0), (' ', 1.0), ('6', 1.0), ('.', 1.0), (' ', 1.0), ('7', 1.0), ('.', 1.0), (' ', 1.0), ('8', 1.0), ('.', 1.0), (' ', 1.0)]</t>
         </is>
       </c>
       <c r="L49" t="n">
@@ -2815,7 +2802,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>What is the location of CFMJ?</t>
+          <t>W6hat i"s the location% of CFMJ?</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2828,31 +2815,29 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>What is the location of CFMJ? Answer: CFMJ is located at 550 Bay Street, Toronto, Ontario, M5G 2M9.
-What is the</t>
+          <t xml:space="preserve">W6hat i"s the location% of CFMJ? Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Answer: CFMJ is located at 550 Bay Street, Toronto, Ontario, M5G 2M9.
-What is the</t>
+          <t xml:space="preserve">Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="G50" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="H50" t="n">
-        <v>0.9460576772689819</v>
+        <v>1</v>
       </c>
       <c r="I50" t="n">
-        <v>0.6931471824645996</v>
+        <v>-0</v>
       </c>
       <c r="J50" t="b">
         <v>0</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>[(' CF', 1.0), ('MJ', 1.0), (' is', 1.0), (' located', 1.0), (' at', 1.0), (' ', 1.0), ('550', 0.5), (' Bay', 1.0), (' Street', 1.0), (',', 1.0), (' Toronto', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' M', 0.5), ('5', 1.0), ('G', 1.0), (' ', 1.0), ('2', 1.0), ('M', 1.0), ('9', 1.0), ('.\n', 1.0), ('What', 1.0), (' is', 1.0), (' the', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' ', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('4', 1.0), ('.', 1.0), (' ', 1.0), ('5', 1.0), ('.', 1.0), (' ', 1.0), ('6', 1.0), ('.', 1.0), (' ', 1.0), ('7', 1.0), ('.', 1.0), (' ', 1.0), ('8', 1.0), ('.', 1.0), (' ', 1.0)]</t>
         </is>
       </c>
       <c r="L50" t="n">
@@ -2865,7 +2850,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>What is the location of CFMJ?</t>
+          <t>W6hat i"s the location% of CFMJ?</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2878,31 +2863,29 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>What is the location of CFMJ? Answer: CFMJ is located at 101 The East Mall, Toronto, Ontario, M9B 6K1.
-What is</t>
+          <t xml:space="preserve">W6hat i"s the location% of CFMJ? Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Answer: CFMJ is located at 101 The East Mall, Toronto, Ontario, M9B 6K1.
-What is</t>
+          <t xml:space="preserve">Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="G51" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H51" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I51" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J51" t="b">
         <v>0</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>[(' CF', 1.0), ('MJ', 1.0), (' is', 1.0), (' located', 1.0), (' at', 1.0), (' ', 1.0), ('101', 0.5), (' The', 1.0), (' East', 1.0), (' Mall', 1.0), (',', 1.0), (' Toronto', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' M', 1.0), ('9', 1.0), ('B', 1.0), (' ', 1.0), ('6', 1.0), ('K', 1.0), ('1', 1.0), ('.\n', 1.0), ('What', 1.0), (' is', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' ', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('4', 1.0), ('.', 1.0), (' ', 1.0), ('5', 1.0), ('.', 1.0), (' ', 1.0), ('6', 1.0), ('.', 1.0), (' ', 1.0), ('7', 1.0), ('.', 1.0), (' ', 1.0), ('8', 1.0), ('.', 1.0), (' ', 1.0)]</t>
         </is>
       </c>
       <c r="L51" t="n">
@@ -2915,7 +2898,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>What is the location of Amos Anderson Art Museum?</t>
+          <t>.What is the locatio7n of Amo~s Anderson Art Museum?</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2928,12 +2911,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>What is the location of Amos Anderson Art Museum? Answer: Amos Anderson Art Museum is located in Helsinki, Finland. Amos Anderson Art Museum is located in Helsinki, Finland. Am</t>
+          <t>.What is the locatio7n of Amo~s Anderson Art Museum? Answer: 1. What is the location of Amos Anderson Art Museum? 2. What is the location of Amos Anderson</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Answer: Amos Anderson Art Museum is located in Helsinki, Finland</t>
+          <t>Answer: 1. What is the location of Amos Anderson Art Museum? 2. What is the location of Amos Anderson</t>
         </is>
       </c>
       <c r="G52" t="n">
@@ -2946,15 +2929,15 @@
         <v>-0</v>
       </c>
       <c r="J52" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>[(' Am', 1.0), ('os', 1.0), (' Anderson', 1.0), (' Art', 1.0), (' Museum', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Helsinki', 1.0), (',', 1.0), (' Finland', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' What', 1.0), (' is', 1.0), (' the', 1.0), (' location', 1.0), (' of', 1.0), (' Am', 1.0), ('os', 1.0), (' Anderson', 1.0), (' Art', 1.0), (' Museum', 1.0), ('?', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' What', 1.0), (' is', 1.0), (' the', 1.0), (' location', 1.0), (' of', 1.0), (' Am', 1.0), ('os', 1.0), (' Anderson', 1.0)]</t>
         </is>
       </c>
       <c r="L52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -2963,7 +2946,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>What is the location of Amos Anderson Art Museum?</t>
+          <t>.What is the locatio7n of Amo~s Anderson Art Museum?</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2976,12 +2959,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>What is the location of Amos Anderson Art Museum? Answer: Amos Anderson Art Museum is located in Helsinki, Finland. Amos Anderson Art Museum is located in Helsinki, Finland. Am</t>
+          <t>.What is the locatio7n of Amo~s Anderson Art Museum? Answer: 1. What is the location of Amos Anderson Art Museum? 2. What is the location of Amos Anderson</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Answer: Amos Anderson Art Museum is located in Helsinki, Finland</t>
+          <t>Answer: 1. What is the location of Amos Anderson Art Museum? 2. What is the location of Amos Anderson</t>
         </is>
       </c>
       <c r="G53" t="n">
@@ -2994,15 +2977,15 @@
         <v>-0</v>
       </c>
       <c r="J53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>[(' Am', 1.0), ('os', 1.0), (' Anderson', 1.0), (' Art', 1.0), (' Museum', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Helsinki', 1.0), (',', 1.0), (' Finland', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' What', 1.0), (' is', 1.0), (' the', 1.0), (' location', 1.0), (' of', 1.0), (' Am', 1.0), ('os', 1.0), (' Anderson', 1.0), (' Art', 1.0), (' Museum', 1.0), ('?', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' What', 1.0), (' is', 1.0), (' the', 1.0), (' location', 1.0), (' of', 1.0), (' Am', 1.0), ('os', 1.0), (' Anderson', 1.0)]</t>
         </is>
       </c>
       <c r="L53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -3011,7 +2994,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>What is the location of Amos Anderson Art Museum?</t>
+          <t>.What is the locatio7n of Amo~s Anderson Art Museum?</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3024,12 +3007,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>What is the location of Amos Anderson Art Museum? Answer: Amos Anderson Art Museum is located in Helsinki, Finland. The museum is located in the city center, near the Helsinki Cathedral</t>
+          <t>.What is the locatio7n of Amo~s Anderson Art Museum? Answer: 1. What is the location of Amos Anderson Art Museum? 2. What is the location of Amos Anderson</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Answer: Amos Anderson Art Museum is located in Helsinki, Finland</t>
+          <t>Answer: 1. What is the location of Amos Anderson Art Museum? 2. What is the location of Amos Anderson</t>
         </is>
       </c>
       <c r="G54" t="n">
@@ -3042,15 +3025,15 @@
         <v>-0</v>
       </c>
       <c r="J54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>[(' Am', 1.0), ('os', 1.0), (' Anderson', 1.0), (' Art', 1.0), (' Museum', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Helsinki', 1.0), (',', 1.0), (' Finland', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' What', 1.0), (' is', 1.0), (' the', 1.0), (' location', 1.0), (' of', 1.0), (' Am', 1.0), ('os', 1.0), (' Anderson', 1.0), (' Art', 1.0), (' Museum', 1.0), ('?', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' What', 1.0), (' is', 1.0), (' the', 1.0), (' location', 1.0), (' of', 1.0), (' Am', 1.0), ('os', 1.0), (' Anderson', 1.0)]</t>
         </is>
       </c>
       <c r="L54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -3059,7 +3042,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>What is the location of Amos Anderson Art Museum?</t>
+          <t>.What is the locatio7n of Amo~s Anderson Art Museum?</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3072,12 +3055,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>What is the location of Amos Anderson Art Museum? Answer: Amos Anderson Art Museum is located in Helsinki, Finland. Amos Anderson Art Museum is located in Helsinki, Finland. Am</t>
+          <t>.What is the locatio7n of Amo~s Anderson Art Museum? Answer: 1. What is the location of Amos Anderson Art Museum? 2. What is the location of Amos Anderson</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Answer: Amos Anderson Art Museum is located in Helsinki, Finland</t>
+          <t>Answer: 1. What is the location of Amos Anderson Art Museum? 2. What is the location of Amos Anderson</t>
         </is>
       </c>
       <c r="G55" t="n">
@@ -3090,15 +3073,15 @@
         <v>-0</v>
       </c>
       <c r="J55" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>[(' Am', 1.0), ('os', 1.0), (' Anderson', 1.0), (' Art', 1.0), (' Museum', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Helsinki', 1.0), (',', 1.0), (' Finland', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' What', 1.0), (' is', 1.0), (' the', 1.0), (' location', 1.0), (' of', 1.0), (' Am', 1.0), ('os', 1.0), (' Anderson', 1.0), (' Art', 1.0), (' Museum', 1.0), ('?', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' What', 1.0), (' is', 1.0), (' the', 1.0), (' location', 1.0), (' of', 1.0), (' Am', 1.0), ('os', 1.0), (' Anderson', 1.0)]</t>
         </is>
       </c>
       <c r="L55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -3107,7 +3090,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>What is the location of Amos Anderson Art Museum?</t>
+          <t>.What is the locatio7n of Amo~s Anderson Art Museum?</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3120,12 +3103,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>What is the location of Amos Anderson Art Museum? Answer: Amos Anderson Art Museum is located in Helsinki, Finland. The museum is located in the city center, near the Helsinki Cathedral</t>
+          <t>.What is the locatio7n of Amo~s Anderson Art Museum? Answer: 1. What is the location of Amos Anderson Art Museum? 2. What is the location of Amos Anderson</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Answer: Amos Anderson Art Museum is located in Helsinki, Finland</t>
+          <t>Answer: 1. What is the location of Amos Anderson Art Museum? 2. What is the location of Amos Anderson</t>
         </is>
       </c>
       <c r="G56" t="n">
@@ -3138,15 +3121,15 @@
         <v>-0</v>
       </c>
       <c r="J56" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>[(' Am', 1.0), ('os', 1.0), (' Anderson', 1.0), (' Art', 1.0), (' Museum', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Helsinki', 1.0), (',', 1.0), (' Finland', 1.0)]</t>
+          <t>[(' ', 1.0), ('1', 1.0), ('.', 1.0), (' What', 1.0), (' is', 1.0), (' the', 1.0), (' location', 1.0), (' of', 1.0), (' Am', 1.0), ('os', 1.0), (' Anderson', 1.0), (' Art', 1.0), (' Museum', 1.0), ('?', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' What', 1.0), (' is', 1.0), (' the', 1.0), (' location', 1.0), (' of', 1.0), (' Am', 1.0), ('os', 1.0), (' Anderson', 1.0)]</t>
         </is>
       </c>
       <c r="L56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -3155,7 +3138,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>What is the location of Zelenchukskaya?</t>
+          <t>What (is 6the location of Zelenchukskay_a?</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3168,29 +3151,29 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>What is the location of Zelenchukskaya? Answer: Zelenchukskaya is located in Russia (Krasnodarskiy Kray) and time zone Asia/M</t>
+          <t>What (is 6the location of Zelenchukskay_a? Answer: Zelenchukskaya is located in Russia. Coordinates of Zelenchukskaya is: 43.75</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Answer: Zelenchukskaya is located in Russia (Krasnodarskiy Kray) and time zone Asia/M</t>
+          <t>Answer: Zelenchukskaya is located in Russia</t>
         </is>
       </c>
       <c r="G57" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H57" t="n">
-        <v>1</v>
+        <v>0.9330329895019531</v>
       </c>
       <c r="I57" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J57" t="b">
         <v>1</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>[(' Z', 1.0), ('elen', 1.0), ('chu', 1.0), ('ks', 1.0), ('k', 1.0), ('aya', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Russia', 1.0)]</t>
+          <t>[(' Z', 1.0), ('elen', 1.0), ('chu', 1.0), ('ks', 1.0), ('k', 1.0), ('aya', 0.5), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Russia', 1.0)]</t>
         </is>
       </c>
       <c r="L57" t="n">
@@ -3203,7 +3186,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>What is the location of Zelenchukskaya?</t>
+          <t>What (is 6the location of Zelenchukskay_a?</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3216,29 +3199,29 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>What is the location of Zelenchukskaya? Answer: Zelenchukskaya is located in Russia (Krasnodarskiy Kray) and time zone Asia/M</t>
+          <t>What (is 6the location of Zelenchukskay_a? Answer: Zelenchukskaya is located in Russia. Coordinates of Zelenchukskaya is: 43.75</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Answer: Zelenchukskaya is located in Russia (Krasnodarskiy Kray) and time zone Asia/M</t>
+          <t>Answer: Zelenchukskaya is located in Russia</t>
         </is>
       </c>
       <c r="G58" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H58" t="n">
-        <v>1</v>
+        <v>0.9330329895019531</v>
       </c>
       <c r="I58" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J58" t="b">
         <v>1</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>[(' Z', 1.0), ('elen', 1.0), ('chu', 1.0), ('ks', 1.0), ('k', 1.0), ('aya', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Russia', 1.0)]</t>
+          <t>[(' Z', 1.0), ('elen', 1.0), ('chu', 1.0), ('ks', 1.0), ('k', 1.0), ('aya', 0.5), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Russia', 1.0)]</t>
         </is>
       </c>
       <c r="L58" t="n">
@@ -3251,7 +3234,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>What is the location of Zelenchukskaya?</t>
+          <t>What (is 6the location of Zelenchukskay_a?</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3264,29 +3247,29 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>What is the location of Zelenchukskaya? Answer: Zelenchukskaya is located in Russia (Krasnodarskiy Kray) and time zone Asia/M</t>
+          <t>What (is 6the location of Zelenchukskay_a? Answer: Zelenchukskay_a is located in Russia. Coordinates of Zelenchukskay_a is: 43</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Answer: Zelenchukskaya is located in Russia (Krasnodarskiy Kray) and time zone Asia/M</t>
+          <t>Answer: Zelenchukskay_a is located in Russia</t>
         </is>
       </c>
       <c r="G59" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H59" t="n">
-        <v>1</v>
+        <v>0.9389309287071228</v>
       </c>
       <c r="I59" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J59" t="b">
         <v>1</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>[(' Z', 1.0), ('elen', 1.0), ('chu', 1.0), ('ks', 1.0), ('k', 1.0), ('aya', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Russia', 1.0)]</t>
+          <t>[(' Z', 1.0), ('elen', 1.0), ('chu', 1.0), ('ks', 1.0), ('k', 1.0), ('ay', 0.5), ('_a', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Russia', 1.0)]</t>
         </is>
       </c>
       <c r="L59" t="n">
@@ -3299,7 +3282,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>What is the location of Zelenchukskaya?</t>
+          <t>What (is 6the location of Zelenchukskay_a?</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3312,29 +3295,29 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>What is the location of Zelenchukskaya? Answer: Zelenchukskaya is located in Russia (Krasnodarskiy Kray) and time zone Asia/M</t>
+          <t>What (is 6the location of Zelenchukskay_a? Answer: Zelenchukskay_a is located in Russia. Coordinates of Zelenchukskay_a is: 43</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Answer: Zelenchukskaya is located in Russia (Krasnodarskiy Kray) and time zone Asia/M</t>
+          <t>Answer: Zelenchukskay_a is located in Russia</t>
         </is>
       </c>
       <c r="G60" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H60" t="n">
-        <v>1</v>
+        <v>0.9389309287071228</v>
       </c>
       <c r="I60" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J60" t="b">
         <v>1</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>[(' Z', 1.0), ('elen', 1.0), ('chu', 1.0), ('ks', 1.0), ('k', 1.0), ('aya', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Russia', 1.0)]</t>
+          <t>[(' Z', 1.0), ('elen', 1.0), ('chu', 1.0), ('ks', 1.0), ('k', 1.0), ('ay', 0.5), ('_a', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Russia', 1.0)]</t>
         </is>
       </c>
       <c r="L60" t="n">
@@ -3347,7 +3330,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>What is the location of Zelenchukskaya?</t>
+          <t>What (is 6the location of Zelenchukskay_a?</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3360,29 +3343,29 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>What is the location of Zelenchukskaya? Answer: Zelenchukskaya is located in Russia (Krasnodarskiy Kray) and time zone Asia/M</t>
+          <t>What (is 6the location of Zelenchukskay_a? Answer: Zelenchukskaya is located in Russia. Coordinates of Zelenchukskaya is: 43.75</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Answer: Zelenchukskaya is located in Russia (Krasnodarskiy Kray) and time zone Asia/M</t>
+          <t>Answer: Zelenchukskaya is located in Russia</t>
         </is>
       </c>
       <c r="G61" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H61" t="n">
-        <v>1</v>
+        <v>0.9330329895019531</v>
       </c>
       <c r="I61" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J61" t="b">
         <v>1</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>[(' Z', 1.0), ('elen', 1.0), ('chu', 1.0), ('ks', 1.0), ('k', 1.0), ('aya', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Russia', 1.0)]</t>
+          <t>[(' Z', 1.0), ('elen', 1.0), ('chu', 1.0), ('ks', 1.0), ('k', 1.0), ('aya', 0.5), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Russia', 1.0)]</t>
         </is>
       </c>
       <c r="L61" t="n">
@@ -3395,7 +3378,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>What is the location of Santo Stefano d'Aveto?</t>
+          <t>What =is the location of Santo Ste"fano d'Avet2o?</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3408,29 +3391,29 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>What is the location of Santo Stefano d'Aveto? Answer: Santo Stefano d'Aveto is located in Italy (Emilia-Romagna) and time zone Europe/Rome.</t>
+          <t>What =is the location of Santo Ste"fano d'Avet2o? Answer: Santo Stefano d'Aveto is located in the province of Genoa, Liguria region, Italy. The coordinates of</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Answer: Santo Stefano d'Aveto is located in Italy (Emilia-Romagna) and time zone Europe/Rome</t>
+          <t>Answer: Santo Stefano d'Aveto is located in the province of Genoa, Liguria region, Italy</t>
         </is>
       </c>
       <c r="G62" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H62" t="n">
-        <v>1</v>
+        <v>0.9675318002700806</v>
       </c>
       <c r="I62" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J62" t="b">
         <v>1</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>[(' Santo', 1.0), (' Stef', 1.0), ('ano', 1.0), (' d', 1.0), ("'", 1.0), ('Av', 1.0), ('eto', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Italy', 1.0)]</t>
+          <t>[(' Santo', 1.0), (' Stef', 1.0), ('ano', 1.0), (' d', 1.0), ("'", 1.0), ('Av', 1.0), ('eto', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' province', 1.0), (' of', 1.0), (' Gen', 1.0), ('oa', 1.0), (',', 1.0), (' Lig', 1.0), ('uria', 1.0), (' region', 0.5), (',', 1.0), (' Italy', 1.0)]</t>
         </is>
       </c>
       <c r="L62" t="n">
@@ -3443,7 +3426,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>What is the location of Santo Stefano d'Aveto?</t>
+          <t>What =is the location of Santo Ste"fano d'Avet2o?</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3456,29 +3439,29 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>What is the location of Santo Stefano d'Aveto? Answer: Santo Stefano d'Aveto is located in Italy (Emilia-Romagna) and time zone of Santo Stefano</t>
+          <t>What =is the location of Santo Ste"fano d'Avet2o? Answer: Santo Stefano d'Aveto is located in the province of Genoa, Liguria region, Italy. The coordinates of</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Answer: Santo Stefano d'Aveto is located in Italy (Emilia-Romagna) and time zone of Santo Stefano</t>
+          <t>Answer: Santo Stefano d'Aveto is located in the province of Genoa, Liguria region, Italy</t>
         </is>
       </c>
       <c r="G63" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H63" t="n">
-        <v>1</v>
+        <v>0.9675318002700806</v>
       </c>
       <c r="I63" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J63" t="b">
         <v>1</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>[(' Santo', 1.0), (' Stef', 1.0), ('ano', 1.0), (' d', 1.0), ("'", 1.0), ('Av', 1.0), ('eto', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Italy', 1.0)]</t>
+          <t>[(' Santo', 1.0), (' Stef', 1.0), ('ano', 1.0), (' d', 1.0), ("'", 1.0), ('Av', 1.0), ('eto', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' province', 1.0), (' of', 1.0), (' Gen', 1.0), ('oa', 1.0), (',', 1.0), (' Lig', 1.0), ('uria', 1.0), (' region', 0.5), (',', 1.0), (' Italy', 1.0)]</t>
         </is>
       </c>
       <c r="L63" t="n">
@@ -3491,7 +3474,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>What is the location of Santo Stefano d'Aveto?</t>
+          <t>What =is the location of Santo Ste"fano d'Avet2o?</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3504,29 +3487,29 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>What is the location of Santo Stefano d'Aveto? Answer: Santo Stefano d'Aveto is located in Italy (Emilia-Romagna) and time zone Europe/Rome.</t>
+          <t>What =is the location of Santo Ste"fano d'Avet2o? Answer: Santo Stefano d'Aveto is located in the province of Genoa, Liguria region, Italy. The coordinates of</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Answer: Santo Stefano d'Aveto is located in Italy (Emilia-Romagna) and time zone Europe/Rome</t>
+          <t>Answer: Santo Stefano d'Aveto is located in the province of Genoa, Liguria region, Italy</t>
         </is>
       </c>
       <c r="G64" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H64" t="n">
-        <v>1</v>
+        <v>0.9675318002700806</v>
       </c>
       <c r="I64" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J64" t="b">
         <v>1</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>[(' Santo', 1.0), (' Stef', 1.0), ('ano', 1.0), (' d', 1.0), ("'", 1.0), ('Av', 1.0), ('eto', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Italy', 1.0)]</t>
+          <t>[(' Santo', 1.0), (' Stef', 1.0), ('ano', 1.0), (' d', 1.0), ("'", 1.0), ('Av', 1.0), ('eto', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' province', 1.0), (' of', 1.0), (' Gen', 1.0), ('oa', 1.0), (',', 1.0), (' Lig', 1.0), ('uria', 1.0), (' region', 0.5), (',', 1.0), (' Italy', 1.0)]</t>
         </is>
       </c>
       <c r="L64" t="n">
@@ -3539,7 +3522,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>What is the location of Santo Stefano d'Aveto?</t>
+          <t>What =is the location of Santo Ste"fano d'Avet2o?</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3552,29 +3535,29 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>What is the location of Santo Stefano d'Aveto? Answer: Santo Stefano d'Aveto is located in Italy (Emilia-Romagna) and time zone Europe/Rome.</t>
+          <t>What =is the location of Santo Ste"fano d'Avet2o? Answer: Santo Stefano d'Aveto is located in the province of Genoa, Liguria, Italy. The town is located</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Answer: Santo Stefano d'Aveto is located in Italy (Emilia-Romagna) and time zone Europe/Rome</t>
+          <t>Answer: Santo Stefano d'Aveto is located in the province of Genoa, Liguria, Italy</t>
         </is>
       </c>
       <c r="G65" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H65" t="n">
-        <v>1</v>
+        <v>0.9659363031387329</v>
       </c>
       <c r="I65" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J65" t="b">
         <v>1</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>[(' Santo', 1.0), (' Stef', 1.0), ('ano', 1.0), (' d', 1.0), ("'", 1.0), ('Av', 1.0), ('eto', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Italy', 1.0)]</t>
+          <t>[(' Santo', 1.0), (' Stef', 1.0), ('ano', 1.0), (' d', 1.0), ("'", 1.0), ('Av', 1.0), ('eto', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' province', 1.0), (' of', 1.0), (' Gen', 1.0), ('oa', 1.0), (',', 1.0), (' Lig', 1.0), ('uria', 1.0), (',', 0.5), (' Italy', 1.0)]</t>
         </is>
       </c>
       <c r="L65" t="n">
@@ -3587,7 +3570,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>What is the location of Santo Stefano d'Aveto?</t>
+          <t>What =is the location of Santo Ste"fano d'Avet2o?</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3600,29 +3583,29 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>What is the location of Santo Stefano d'Aveto? Answer: Santo Stefano d'Aveto is located in Italy (Emilia-Romagna) and time zone of Santo Stefano</t>
+          <t>What =is the location of Santo Ste"fano d'Avet2o? Answer: Santo Stefano d'Aveto is located in the province of Genoa, Liguria, Italy. The town is situated</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Answer: Santo Stefano d'Aveto is located in Italy (Emilia-Romagna) and time zone of Santo Stefano</t>
+          <t>Answer: Santo Stefano d'Aveto is located in the province of Genoa, Liguria, Italy</t>
         </is>
       </c>
       <c r="G66" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H66" t="n">
-        <v>1</v>
+        <v>0.9659363031387329</v>
       </c>
       <c r="I66" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J66" t="b">
         <v>1</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>[(' Santo', 1.0), (' Stef', 1.0), ('ano', 1.0), (' d', 1.0), ("'", 1.0), ('Av', 1.0), ('eto', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' Italy', 1.0)]</t>
+          <t>[(' Santo', 1.0), (' Stef', 1.0), ('ano', 1.0), (' d', 1.0), ("'", 1.0), ('Av', 1.0), ('eto', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' province', 1.0), (' of', 1.0), (' Gen', 1.0), ('oa', 1.0), (',', 1.0), (' Lig', 1.0), ('uria', 1.0), (',', 0.5), (' Italy', 1.0)]</t>
         </is>
       </c>
       <c r="L66" t="n">
@@ -3635,7 +3618,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>What is the location of SooToday.com?</t>
+          <t>What 6is the= loca0tion of SooToday.com?</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3648,8 +3631,8 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>What is the location of SooToday.com? Answer: Sault Ste. Marie, Ontario, Canada.
-What is the location of SooToday.com? Answer: Sault Ste</t>
+          <t>What 6is the= loca0tion of SooToday.com? Answer: Sault Ste. Marie, Ontario, Canada
+What is the= location of SooToday.com? Answer: Sault</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3658,24 +3641,24 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H67" t="n">
-        <v>1</v>
+        <v>0.9258747100830078</v>
       </c>
       <c r="I67" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J67" t="b">
         <v>1</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>[(' S', 1.0), ('ault', 1.0), (' Ste', 1.0), ('.', 1.0), (' Marie', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' Canada', 1.0)]</t>
+          <t>[(' S', 0.5), ('ault', 1.0), (' Ste', 1.0), ('.', 1.0), (' Marie', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' Canada', 1.0)]</t>
         </is>
       </c>
       <c r="L67" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="68">
@@ -3684,7 +3667,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>What is the location of SooToday.com?</t>
+          <t>What 6is the= loca0tion of SooToday.com?</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3697,8 +3680,8 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>What is the location of SooToday.com? Answer: Sault Ste. Marie, Ontario, Canada.
-What is the postal code of SooToday.com? Answer: P6</t>
+          <t>What 6is the= loca0tion of SooToday.com? Answer: Sault Ste. Marie, Ontario, Canada
+What is the= location of SooToday.com? Answer: Sault</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3707,24 +3690,24 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H68" t="n">
-        <v>1</v>
+        <v>0.9258747100830078</v>
       </c>
       <c r="I68" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J68" t="b">
         <v>1</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>[(' S', 1.0), ('ault', 1.0), (' Ste', 1.0), ('.', 1.0), (' Marie', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' Canada', 1.0)]</t>
+          <t>[(' S', 0.5), ('ault', 1.0), (' Ste', 1.0), ('.', 1.0), (' Marie', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' Canada', 1.0)]</t>
         </is>
       </c>
       <c r="L68" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="69">
@@ -3733,7 +3716,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>What is the location of SooToday.com?</t>
+          <t>What 6is the= loca0tion of SooToday.com?</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3746,8 +3729,8 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>What is the location of SooToday.com? Answer: Sault Ste. Marie, Ontario, Canada.
-What is the location of SooToday.com? Answer: Sault Ste</t>
+          <t>What 6is the= loca0tion of SooToday.com? Answer: Sault Ste. Marie, Ontario, Canada.
+What is the= location of SooToday.com? Answer: Sault</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3756,24 +3739,24 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H69" t="n">
-        <v>1</v>
+        <v>0.9258747100830078</v>
       </c>
       <c r="I69" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J69" t="b">
         <v>1</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>[(' S', 1.0), ('ault', 1.0), (' Ste', 1.0), ('.', 1.0), (' Marie', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' Canada', 1.0)]</t>
+          <t>[(' S', 0.5), ('ault', 1.0), (' Ste', 1.0), ('.', 1.0), (' Marie', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' Canada', 1.0)]</t>
         </is>
       </c>
       <c r="L69" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="70">
@@ -3782,7 +3765,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>What is the location of SooToday.com?</t>
+          <t>What 6is the= loca0tion of SooToday.com?</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3795,8 +3778,8 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>What is the location of SooToday.com? Answer: Sault Ste. Marie, Ontario, Canada.
-What is the location of SooToday.com? Answer: Sault Ste</t>
+          <t>What 6is the= loca0tion of SooToday.com? Answer: Sault Ste. Marie, Ontario, Canada.
+What is the= location of SooToday.com? Answer: Sault</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3805,24 +3788,24 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H70" t="n">
-        <v>1</v>
+        <v>0.9258747100830078</v>
       </c>
       <c r="I70" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J70" t="b">
         <v>1</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>[(' S', 1.0), ('ault', 1.0), (' Ste', 1.0), ('.', 1.0), (' Marie', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' Canada', 1.0)]</t>
+          <t>[(' S', 0.5), ('ault', 1.0), (' Ste', 1.0), ('.', 1.0), (' Marie', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' Canada', 1.0)]</t>
         </is>
       </c>
       <c r="L70" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="71">
@@ -3831,7 +3814,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>What is the location of SooToday.com?</t>
+          <t>What 6is the= loca0tion of SooToday.com?</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3844,34 +3827,33 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>What is the location of SooToday.com? Answer: Sault Ste. Marie, Ontario, Canada.
-What is the location of SooToday.com? Answer: Sault Ste</t>
+          <t xml:space="preserve">What 6is the= loca0tion of SooToday.com? Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Answer: Sault Ste. Marie, Ontario, Canada</t>
+          <t xml:space="preserve">Answer: 1. 2. 3. 4. 5. 6. 7. 8. </t>
         </is>
       </c>
       <c r="G71" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H71" t="n">
-        <v>1</v>
+        <v>0.9726549386978149</v>
       </c>
       <c r="I71" t="n">
-        <v>-0</v>
+        <v>0.3465735912322998</v>
       </c>
       <c r="J71" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>[(' S', 1.0), ('ault', 1.0), (' Ste', 1.0), ('.', 1.0), (' Marie', 1.0), (',', 1.0), (' Ontario', 1.0), (',', 1.0), (' Canada', 1.0)]</t>
+          <t>[(' ', 0.5), ('1', 1.0), ('.', 1.0), (' ', 1.0), ('2', 1.0), ('.', 1.0), (' ', 1.0), ('3', 1.0), ('.', 1.0), (' ', 1.0), ('4', 1.0), ('.', 1.0), (' ', 1.0), ('5', 1.0), ('.', 1.0), (' ', 1.0), ('6', 1.0), ('.', 1.0), (' ', 1.0), ('7', 1.0), ('.', 1.0), (' ', 1.0), ('8', 1.0), ('.', 1.0), (' ', 1.0)]</t>
         </is>
       </c>
       <c r="L71" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="72">
@@ -3880,7 +3862,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>What is the location of Sena Medal?</t>
+          <t>What i&lt;s the\ location 0of Sena Medal?</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3893,34 +3875,33 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>What is the location of Sena Medal? Answer: Sena Medal is located in India (Asia) and the postal code of Sena Medal is 110010.
-What is</t>
+          <t>What i&lt;s the\ location 0of Sena Medal? Answer: (1) On the left breast, in a horizontal line with the 2nd Star. (2) On the left</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Answer: Sena Medal is located in India (Asia) and the postal code of Sena Medal is 110010</t>
+          <t>Answer: (1) On the left breast, in a horizontal line with the 2nd Star. (2) On the left</t>
         </is>
       </c>
       <c r="G72" t="n">
-        <v>0.5</v>
+        <v>0.1943250000476837</v>
       </c>
       <c r="H72" t="n">
-        <v>0.9057236313819885</v>
+        <v>0.9365719556808472</v>
       </c>
       <c r="I72" t="n">
-        <v>0.3465735912322998</v>
+        <v>0.8889715671539307</v>
       </c>
       <c r="J72" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>[(' Sen', 1.0), ('a', 1.0), (' Medal', 1.0), (' is', 1.0), (' located', 0.5), (' in', 1.0), (' India', 1.0)]</t>
+          <t>[(' (', 1.0), ('1', 1.0), (')', 1.0), (' On', 0.7773), (' the', 1.0), (' left', 1.0), (' breast', 0.5), (',', 1.0), (' in', 1.0), (' a', 1.0), (' horizontal', 1.0), (' line', 1.0), (' with', 1.0), (' the', 1.0), (' ', 1.0), ('2', 0.5), ('nd', 1.0), (' Star', 1.0), ('.', 1.0), (' (', 1.0), ('2', 1.0), (')', 1.0), (' On', 1.0), (' the', 1.0), (' left', 1.0)]</t>
         </is>
       </c>
       <c r="L72" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -3929,7 +3910,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>What is the location of Sena Medal?</t>
+          <t>What i&lt;s the\ location 0of Sena Medal?</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3942,34 +3923,33 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>What is the location of Sena Medal? Answer: Sena Medal is located in India (Asia) and the postal code of Sena Medal is 110010.
-What is</t>
+          <t>What i&lt;s the\ location 0of Sena Medal? Answer: (1) On the left side of the chest. (2) On the right side of the chest. (3)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Answer: Sena Medal is located in India (Asia) and the postal code of Sena Medal is 110010</t>
+          <t>Answer: (1) On the left side of the chest. (2) On the right side of the chest. (3)</t>
         </is>
       </c>
       <c r="G73" t="n">
-        <v>0.5</v>
+        <v>0.3886500000953674</v>
       </c>
       <c r="H73" t="n">
-        <v>0.9057236313819885</v>
+        <v>0.9629025459289551</v>
       </c>
       <c r="I73" t="n">
-        <v>0.3465735912322998</v>
+        <v>0.5423979759216309</v>
       </c>
       <c r="J73" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>[(' Sen', 1.0), ('a', 1.0), (' Medal', 1.0), (' is', 1.0), (' located', 0.5), (' in', 1.0), (' India', 1.0)]</t>
+          <t>[(' (', 1.0), ('1', 1.0), (')', 1.0), (' On', 0.7773), (' the', 1.0), (' left', 1.0), (' side', 0.5), (' of', 1.0), (' the', 1.0), (' chest', 1.0), ('.', 1.0), (' (', 1.0), ('2', 1.0), (')', 1.0), (' On', 1.0), (' the', 1.0), (' right', 1.0), (' side', 1.0), (' of', 1.0), (' the', 1.0), (' chest', 1.0), ('.', 1.0), (' (', 1.0), ('3', 1.0), (')', 1.0)]</t>
         </is>
       </c>
       <c r="L73" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -3978,7 +3958,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>What is the location of Sena Medal?</t>
+          <t>What i&lt;s the\ location 0of Sena Medal?</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3991,34 +3971,33 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>What is the location of Sena Medal? Answer: Sena Medal is located in India (Asia) and the postal code of Sena Medal is 110010.
-What is</t>
+          <t>What i&lt;s the\ location 0of Sena Medal? Answer: (1) On the left breast, in a horizontal line with the 2nd Star. (2) On the left</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Answer: Sena Medal is located in India (Asia) and the postal code of Sena Medal is 110010</t>
+          <t>Answer: (1) On the left breast, in a horizontal line with the 2nd Star. (2) On the left</t>
         </is>
       </c>
       <c r="G74" t="n">
-        <v>0.5</v>
+        <v>0.1943250000476837</v>
       </c>
       <c r="H74" t="n">
-        <v>0.9057236313819885</v>
+        <v>0.9365719556808472</v>
       </c>
       <c r="I74" t="n">
-        <v>0.3465735912322998</v>
+        <v>0.8889715671539307</v>
       </c>
       <c r="J74" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>[(' Sen', 1.0), ('a', 1.0), (' Medal', 1.0), (' is', 1.0), (' located', 0.5), (' in', 1.0), (' India', 1.0)]</t>
+          <t>[(' (', 1.0), ('1', 1.0), (')', 1.0), (' On', 0.7773), (' the', 1.0), (' left', 1.0), (' breast', 0.5), (',', 1.0), (' in', 1.0), (' a', 1.0), (' horizontal', 1.0), (' line', 1.0), (' with', 1.0), (' the', 1.0), (' ', 1.0), ('2', 0.5), ('nd', 1.0), (' Star', 1.0), ('.', 1.0), (' (', 1.0), ('2', 1.0), (')', 1.0), (' On', 1.0), (' the', 1.0), (' left', 1.0)]</t>
         </is>
       </c>
       <c r="L74" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -4027,7 +4006,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>What is the location of Sena Medal?</t>
+          <t>What i&lt;s the\ location 0of Sena Medal?</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -4040,33 +4019,33 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>What is the location of Sena Medal? Answer: Sena Medal is awarded for gallantry in the face of the enemy. It is awarded to officers and other ranks of the</t>
+          <t>What i&lt;s the\ location 0of Sena Medal? Answer: (1) On the left side of the chest. (2) On the right side of the chest. (3)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Answer: Sena Medal is awarded for gallantry in the face of the enemy. It is awarded to officers and other ranks of the</t>
+          <t>Answer: (1) On the left side of the chest. (2) On the right side of the chest. (3)</t>
         </is>
       </c>
       <c r="G75" t="n">
-        <v>0.09716250747442245</v>
+        <v>0.3886500000953674</v>
       </c>
       <c r="H75" t="n">
-        <v>0.9109613299369812</v>
+        <v>0.9629025459289551</v>
       </c>
       <c r="I75" t="n">
-        <v>1.23554515838623</v>
+        <v>0.5423979759216309</v>
       </c>
       <c r="J75" t="b">
         <v>0</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>[(' Sen', 1.0), ('a', 1.0), (' Medal', 1.0), (' is', 1.0), (' awarded', 0.5), (' for', 1.0), (' gall', 0.5), ('antry', 1.0), (' in', 0.7773), (' the', 1.0), (' face', 1.0), (' of', 1.0), (' the', 1.0), (' enemy', 1.0), ('.', 0.5), (' It', 1.0), (' is', 1.0), (' awarded', 1.0), (' to', 1.0), (' officers', 1.0), (' and', 1.0), (' other', 1.0), (' ranks', 1.0), (' of', 1.0), (' the', 1.0)]</t>
+          <t>[(' (', 1.0), ('1', 1.0), (')', 1.0), (' On', 0.7773), (' the', 1.0), (' left', 1.0), (' side', 0.5), (' of', 1.0), (' the', 1.0), (' chest', 1.0), ('.', 1.0), (' (', 1.0), ('2', 1.0), (')', 1.0), (' On', 1.0), (' the', 1.0), (' right', 1.0), (' side', 1.0), (' of', 1.0), (' the', 1.0), (' chest', 1.0), ('.', 1.0), (' (', 1.0), ('3', 1.0), (')', 1.0)]</t>
         </is>
       </c>
       <c r="L75" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -4075,7 +4054,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>What is the location of Sena Medal?</t>
+          <t>What i&lt;s the\ location 0of Sena Medal?</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -4088,12 +4067,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>What is the location of Sena Medal? Answer: Sena Medal is awarded for acts of gallantry and distinguished service in the field. The medal is awarded to officers and other</t>
+          <t>What i&lt;s the\ location 0of Sena Medal? Answer: (1) On the left breast, in a horizontal line with the 1914 Star. (2) On the left</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Answer: Sena Medal is awarded for acts of gallantry and distinguished service in the field. The medal is awarded to officers and other</t>
+          <t>Answer: (1) On the left breast, in a horizontal line with the 1914 Star. (2) On the left</t>
         </is>
       </c>
       <c r="G76" t="n">
@@ -4110,11 +4089,11 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>[(' Sen', 1.0), ('a', 1.0), (' Medal', 1.0), (' is', 1.0), (' awarded', 0.5), (' for', 1.0), (' acts', 0.5), (' of', 1.0), (' gall', 1.0), ('antry', 1.0), (' and', 0.7773), (' distinguished', 1.0), (' service', 1.0), (' in', 1.0), (' the', 1.0), (' field', 1.0), ('.', 1.0), (' The', 1.0), (' medal', 1.0), (' is', 1.0), (' awarded', 1.0), (' to', 1.0), (' officers', 1.0), (' and', 1.0), (' other', 1.0)]</t>
+          <t>[(' (', 1.0), ('1', 1.0), (')', 1.0), (' On', 0.7773), (' the', 1.0), (' left', 1.0), (' breast', 0.5), (',', 1.0), (' in', 1.0), (' a', 1.0), (' horizontal', 1.0), (' line', 1.0), (' with', 1.0), (' the', 1.0), (' ', 1.0), ('191', 0.5), ('4', 1.0), (' Star', 1.0), ('.', 1.0), (' (', 1.0), ('2', 1.0), (')', 1.0), (' On', 1.0), (' the', 1.0), (' left', 1.0)]</t>
         </is>
       </c>
       <c r="L76" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -4123,7 +4102,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>What is the location of Lake Caliraya?</t>
+          <t>W@hat is ^the locati+on of Lake Caliraya?</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -4136,7 +4115,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the location of Lake Caliraya? Answer: Lake Caliraya is located in the province of Laguna, Philippines. It is a man-made lake that was created in </t>
+          <t>W@hat is ^the locati+on of Lake Caliraya? Answer: Lake Caliraya is located in the province of Laguna, Philippines. It is a man-made lake created by the construction of</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4171,7 +4150,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>What is the location of Lake Caliraya?</t>
+          <t>W@hat is ^the locati+on of Lake Caliraya?</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -4184,7 +4163,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the location of Lake Caliraya? Answer: Lake Caliraya is located in the province of Laguna, Philippines. It is a man-made lake that was created in </t>
+          <t>W@hat is ^the locati+on of Lake Caliraya? Answer: Lake Caliraya is located in the province of Laguna, Philippines. It is a man-made lake created by the construction of</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -4219,7 +4198,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>What is the location of Lake Caliraya?</t>
+          <t>W@hat is ^the locati+on of Lake Caliraya?</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4232,7 +4211,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the location of Lake Caliraya? Answer: Lake Caliraya is located in the province of Laguna, Philippines. It is a man-made lake that was created in </t>
+          <t>W@hat is ^the locati+on of Lake Caliraya? Answer: Lake Caliraya is located in the province of Laguna, Philippines. It is a man-made lake created by the construction of</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4267,7 +4246,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>What is the location of Lake Caliraya?</t>
+          <t>W@hat is ^the locati+on of Lake Caliraya?</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4280,7 +4259,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the location of Lake Caliraya? Answer: Lake Caliraya is located in the province of Laguna, Philippines. It is a man-made lake that was created in </t>
+          <t>W@hat is ^the locati+on of Lake Caliraya? Answer: Lake Caliraya is located in the province of Laguna, Philippines. It is a man-made lake created by the construction of</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4315,7 +4294,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>What is the location of Lake Caliraya?</t>
+          <t>W@hat is ^the locati+on of Lake Caliraya?</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4328,7 +4307,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the location of Lake Caliraya? Answer: Lake Caliraya is located in the province of Laguna, Philippines. It is a man-made lake that was created in </t>
+          <t>W@hat is ^the locati+on of Lake Caliraya? Answer: Lake Caliraya is located in the province of Laguna, Philippines. It is a man-made lake created by the construction of</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4363,7 +4342,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>What is the location of Didymoteicho?</t>
+          <t>)What is the- location of Didym%oteicho?</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4376,13 +4355,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the location of Didymoteicho? Answer: Didymoteicho is located in - Greece (Europe) and the population of the city is 11,896 inhabitants.
-</t>
+          <t>)What is the- location of Didym%oteicho? Answer: Didymoteicho is located in the region of Evros in Greece at 41.33% latitude (from Equator</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Answer: Didymoteicho is located in - Greece (Europe) and the population of the city is 11</t>
+          <t>Answer: Didymoteicho is located in the region of Evros in Greece at 41</t>
         </is>
       </c>
       <c r="G82" t="n">
@@ -4399,7 +4377,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>[(' Did', 1.0), ('ym', 1.0), ('ote', 1.0), ('icho', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' -', 1.0), (' Greece', 1.0)]</t>
+          <t>[(' Did', 1.0), ('ym', 1.0), ('ote', 1.0), ('icho', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' region', 1.0), (' of', 1.0), (' Ev', 1.0), ('ros', 1.0), (' in', 1.0), (' Greece', 1.0), (' at', 1.0), (' ', 1.0), ('41', 1.0)]</t>
         </is>
       </c>
       <c r="L82" t="n">
@@ -4412,7 +4390,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>What is the location of Didymoteicho?</t>
+          <t>)What is the- location of Didym%oteicho?</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4425,13 +4403,12 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the location of Didymoteicho? Answer: Didymoteicho is located in - Greece (Europe) and the population of the city is 10,700 inhabitants.
-</t>
+          <t>)What is the- location of Didym%oteicho? Answer: Didymoteicho is located in the region of Evros in Greece at 41.33% latitude (from Equator</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Answer: Didymoteicho is located in - Greece (Europe) and the population of the city is 10</t>
+          <t>Answer: Didymoteicho is located in the region of Evros in Greece at 41</t>
         </is>
       </c>
       <c r="G83" t="n">
@@ -4448,7 +4425,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>[(' Did', 1.0), ('ym', 1.0), ('ote', 1.0), ('icho', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' -', 1.0), (' Greece', 1.0)]</t>
+          <t>[(' Did', 1.0), ('ym', 1.0), ('ote', 1.0), ('icho', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' region', 1.0), (' of', 1.0), (' Ev', 1.0), ('ros', 1.0), (' in', 1.0), (' Greece', 1.0), (' at', 1.0), (' ', 1.0), ('41', 1.0)]</t>
         </is>
       </c>
       <c r="L83" t="n">
@@ -4461,7 +4438,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>What is the location of Didymoteicho?</t>
+          <t>)What is the- location of Didym%oteicho?</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4474,13 +4451,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the location of Didymoteicho? Answer: Didymoteicho is located in - Greece (Europe) and the population of the city is 10,700 inhabitants.
-</t>
+          <t>)What is the- location of Didym%oteicho? Answer: Didymoteicho is located in the region of Evros in Greece at 41.33% latitude (from Equator</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Answer: Didymoteicho is located in - Greece (Europe) and the population of the city is 10</t>
+          <t>Answer: Didymoteicho is located in the region of Evros in Greece at 41</t>
         </is>
       </c>
       <c r="G84" t="n">
@@ -4497,7 +4473,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>[(' Did', 1.0), ('ym', 1.0), ('ote', 1.0), ('icho', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' -', 1.0), (' Greece', 1.0)]</t>
+          <t>[(' Did', 1.0), ('ym', 1.0), ('ote', 1.0), ('icho', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' region', 1.0), (' of', 1.0), (' Ev', 1.0), ('ros', 1.0), (' in', 1.0), (' Greece', 1.0), (' at', 1.0), (' ', 1.0), ('41', 1.0)]</t>
         </is>
       </c>
       <c r="L84" t="n">
@@ -4510,7 +4486,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>What is the location of Didymoteicho?</t>
+          <t>)What is the- location of Didym%oteicho?</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4523,13 +4499,12 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the location of Didymoteicho? Answer: Didymoteicho is located in - Greece (Europe) and the population of the city is 10,700 inhabitants.
-</t>
+          <t>)What is the- location of Didym%oteicho? Answer: Didymoteicho is located in the region of Evros in Greece at 41.33% latitude (from Equator</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Answer: Didymoteicho is located in - Greece (Europe) and the population of the city is 10</t>
+          <t>Answer: Didymoteicho is located in the region of Evros in Greece at 41</t>
         </is>
       </c>
       <c r="G85" t="n">
@@ -4546,7 +4521,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>[(' Did', 1.0), ('ym', 1.0), ('ote', 1.0), ('icho', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' -', 1.0), (' Greece', 1.0)]</t>
+          <t>[(' Did', 1.0), ('ym', 1.0), ('ote', 1.0), ('icho', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' region', 1.0), (' of', 1.0), (' Ev', 1.0), ('ros', 1.0), (' in', 1.0), (' Greece', 1.0), (' at', 1.0), (' ', 1.0), ('41', 1.0)]</t>
         </is>
       </c>
       <c r="L85" t="n">
@@ -4559,7 +4534,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>What is the location of Didymoteicho?</t>
+          <t>)What is the- location of Didym%oteicho?</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4572,13 +4547,12 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the location of Didymoteicho? Answer: Didymoteicho is located in - Greece (Europe) and the population of the city is 11,896 inhabitants.
-</t>
+          <t>)What is the- location of Didym%oteicho? Answer: Didymoteicho is located in the region of Evros in Greece at 41.33% latitude (from Equator</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Answer: Didymoteicho is located in - Greece (Europe) and the population of the city is 11</t>
+          <t>Answer: Didymoteicho is located in the region of Evros in Greece at 41</t>
         </is>
       </c>
       <c r="G86" t="n">
@@ -4595,7 +4569,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>[(' Did', 1.0), ('ym', 1.0), ('ote', 1.0), ('icho', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' -', 1.0), (' Greece', 1.0)]</t>
+          <t>[(' Did', 1.0), ('ym', 1.0), ('ote', 1.0), ('icho', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' region', 1.0), (' of', 1.0), (' Ev', 1.0), ('ros', 1.0), (' in', 1.0), (' Greece', 1.0), (' at', 1.0), (' ', 1.0), ('41', 1.0)]</t>
         </is>
       </c>
       <c r="L86" t="n">
@@ -4608,7 +4582,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>What is the location of 2004 Indian Ocean earthquake?</t>
+          <t>What is the2 loca6tion of 2004 In(dian Ocean earthquake?</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4621,29 +4595,29 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>What is the location of 2004 Indian Ocean earthquake? Answer: The 2004 Indian Ocean earthquake occurred on December 26, 2004, at 00:58:53 UTC</t>
+          <t>What is the2 loca6tion of 2004 In(dian Ocean earthquake? Answer: The 2004 Indian Ocean earthquake occurred on 26 December 2004 at 00:58:53 UTC. The</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Answer: The 2004 Indian Ocean earthquake occurred on December 26, 2004, at 00:58:53 UTC</t>
+          <t>Answer: The 2004 Indian Ocean earthquake occurred on 26 December 2004 at 00:58:53 UTC. The</t>
         </is>
       </c>
       <c r="G87" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H87" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I87" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J87" t="b">
         <v>0</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>[(' The', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' Indian', 1.0), (' Ocean', 1.0), (' earthquake', 1.0), (' occurred', 1.0), (' on', 1.0), (' December', 0.5), (' ', 1.0), ('26', 1.0), (',', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (',', 1.0), (' at', 1.0), (' ', 1.0), ('00', 1.0), (':', 1.0), ('58', 1.0), (':', 1.0), ('53', 1.0), (' UTC', 1.0)]</t>
+          <t>[(' The', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' Indian', 1.0), (' Ocean', 1.0), (' earthquake', 1.0), (' occurred', 1.0), (' on', 1.0), (' ', 1.0), ('26', 1.0), (' December', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' at', 1.0), (' ', 1.0), ('00', 1.0), (':', 1.0), ('58', 1.0), (':', 1.0), ('53', 1.0), (' UTC', 1.0), ('.', 1.0), (' The', 1.0)]</t>
         </is>
       </c>
       <c r="L87" t="n">
@@ -4656,7 +4630,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>What is the location of 2004 Indian Ocean earthquake?</t>
+          <t>What is the2 loca6tion of 2004 In(dian Ocean earthquake?</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4669,29 +4643,29 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>What is the location of 2004 Indian Ocean earthquake? Answer: The 2004 Indian Ocean earthquake occurred on December 26, 2004, at 00:58:53 UTC</t>
+          <t>What is the2 loca6tion of 2004 In(dian Ocean earthquake? Answer: The 2004 Indian Ocean earthquake occurred on 26 December 2004 at 00:58:53 UTC. The</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Answer: The 2004 Indian Ocean earthquake occurred on December 26, 2004, at 00:58:53 UTC</t>
+          <t>Answer: The 2004 Indian Ocean earthquake occurred on 26 December 2004 at 00:58:53 UTC. The</t>
         </is>
       </c>
       <c r="G88" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H88" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I88" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J88" t="b">
         <v>0</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>[(' The', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' Indian', 1.0), (' Ocean', 1.0), (' earthquake', 1.0), (' occurred', 1.0), (' on', 1.0), (' December', 0.5), (' ', 1.0), ('26', 1.0), (',', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (',', 1.0), (' at', 1.0), (' ', 1.0), ('00', 1.0), (':', 1.0), ('58', 1.0), (':', 1.0), ('53', 1.0), (' UTC', 1.0)]</t>
+          <t>[(' The', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' Indian', 1.0), (' Ocean', 1.0), (' earthquake', 1.0), (' occurred', 1.0), (' on', 1.0), (' ', 1.0), ('26', 1.0), (' December', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' at', 1.0), (' ', 1.0), ('00', 1.0), (':', 1.0), ('58', 1.0), (':', 1.0), ('53', 1.0), (' UTC', 1.0), ('.', 1.0), (' The', 1.0)]</t>
         </is>
       </c>
       <c r="L88" t="n">
@@ -4704,7 +4678,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>What is the location of 2004 Indian Ocean earthquake?</t>
+          <t>What is the2 loca6tion of 2004 In(dian Ocean earthquake?</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4717,7 +4691,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>What is the location of 2004 Indian Ocean earthquake? Answer: The 2004 Indian Ocean earthquake occurred on 26 December 2004 at 00:58:53 UTC. The</t>
+          <t>What is the2 loca6tion of 2004 In(dian Ocean earthquake? Answer: The 2004 Indian Ocean earthquake occurred on 26 December 2004 at 00:58:53 UTC. The</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4726,20 +4700,20 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H89" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I89" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J89" t="b">
         <v>0</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>[(' The', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' Indian', 1.0), (' Ocean', 1.0), (' earthquake', 1.0), (' occurred', 1.0), (' on', 1.0), (' ', 0.5), ('26', 1.0), (' December', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' at', 1.0), (' ', 1.0), ('00', 1.0), (':', 1.0), ('58', 1.0), (':', 1.0), ('53', 1.0), (' UTC', 1.0), ('.', 1.0), (' The', 1.0)]</t>
+          <t>[(' The', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' Indian', 1.0), (' Ocean', 1.0), (' earthquake', 1.0), (' occurred', 1.0), (' on', 1.0), (' ', 1.0), ('26', 1.0), (' December', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' at', 1.0), (' ', 1.0), ('00', 1.0), (':', 1.0), ('58', 1.0), (':', 1.0), ('53', 1.0), (' UTC', 1.0), ('.', 1.0), (' The', 1.0)]</t>
         </is>
       </c>
       <c r="L89" t="n">
@@ -4752,7 +4726,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>What is the location of 2004 Indian Ocean earthquake?</t>
+          <t>What is the2 loca6tion of 2004 In(dian Ocean earthquake?</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4765,29 +4739,29 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>What is the location of 2004 Indian Ocean earthquake? Answer: The 2004 Indian Ocean earthquake occurred on December 26, 2004, at 00:58:53 UTC</t>
+          <t>What is the2 loca6tion of 2004 In(dian Ocean earthquake? Answer: The 2004 Indian Ocean earthquake occurred on 26 December 2004 at 00:58:53 UTC. The</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Answer: The 2004 Indian Ocean earthquake occurred on December 26, 2004, at 00:58:53 UTC</t>
+          <t>Answer: The 2004 Indian Ocean earthquake occurred on 26 December 2004 at 00:58:53 UTC. The</t>
         </is>
       </c>
       <c r="G90" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H90" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I90" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J90" t="b">
         <v>0</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>[(' The', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' Indian', 1.0), (' Ocean', 1.0), (' earthquake', 1.0), (' occurred', 1.0), (' on', 1.0), (' December', 0.5), (' ', 1.0), ('26', 1.0), (',', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (',', 1.0), (' at', 1.0), (' ', 1.0), ('00', 1.0), (':', 1.0), ('58', 1.0), (':', 1.0), ('53', 1.0), (' UTC', 1.0)]</t>
+          <t>[(' The', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' Indian', 1.0), (' Ocean', 1.0), (' earthquake', 1.0), (' occurred', 1.0), (' on', 1.0), (' ', 1.0), ('26', 1.0), (' December', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' at', 1.0), (' ', 1.0), ('00', 1.0), (':', 1.0), ('58', 1.0), (':', 1.0), ('53', 1.0), (' UTC', 1.0), ('.', 1.0), (' The', 1.0)]</t>
         </is>
       </c>
       <c r="L90" t="n">
@@ -4800,7 +4774,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>What is the location of 2004 Indian Ocean earthquake?</t>
+          <t>What is the2 loca6tion of 2004 In(dian Ocean earthquake?</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4813,7 +4787,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>What is the location of 2004 Indian Ocean earthquake? Answer: The 2004 Indian Ocean earthquake occurred on 26 December 2004 at 00:58:53 UTC. The</t>
+          <t>What is the2 loca6tion of 2004 In(dian Ocean earthquake? Answer: The 2004 Indian Ocean earthquake occurred on 26 December 2004 at 00:58:53 UTC. The</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4822,20 +4796,20 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H91" t="n">
-        <v>0.9726549386978149</v>
+        <v>1</v>
       </c>
       <c r="I91" t="n">
-        <v>0.3465735912322998</v>
+        <v>-0</v>
       </c>
       <c r="J91" t="b">
         <v>0</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>[(' The', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' Indian', 1.0), (' Ocean', 1.0), (' earthquake', 1.0), (' occurred', 1.0), (' on', 1.0), (' ', 0.5), ('26', 1.0), (' December', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' at', 1.0), (' ', 1.0), ('00', 1.0), (':', 1.0), ('58', 1.0), (':', 1.0), ('53', 1.0), (' UTC', 1.0), ('.', 1.0), (' The', 1.0)]</t>
+          <t>[(' The', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' Indian', 1.0), (' Ocean', 1.0), (' earthquake', 1.0), (' occurred', 1.0), (' on', 1.0), (' ', 1.0), ('26', 1.0), (' December', 1.0), (' ', 1.0), ('200', 1.0), ('4', 1.0), (' at', 1.0), (' ', 1.0), ('00', 1.0), (':', 1.0), ('58', 1.0), (':', 1.0), ('53', 1.0), (' UTC', 1.0), ('.', 1.0), (' The', 1.0)]</t>
         </is>
       </c>
       <c r="L91" t="n">
@@ -4848,7 +4822,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>What is the location of Fawkner?</t>
+          <t>What is the] loc^ation of `Fawkner?</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4861,12 +4835,12 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>What is the location of Fawkner? Answer: Fawkner is located in the state of Victoria, Australia. The city is located in the northern suburbs of Melbourne, the</t>
+          <t>What is the] loc^ation of `Fawkner? Answer: Fawkner is located in the north of Melbourne, Victoria, Australia. It is a suburb of Melbourne. It is located</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Answer: Fawkner is located in the state of Victoria, Australia</t>
+          <t>Answer: Fawkner is located in the north of Melbourne, Victoria, Australia</t>
         </is>
       </c>
       <c r="G92" t="n">
@@ -4883,7 +4857,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>[(' F', 1.0), ('awk', 1.0), ('ner', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' state', 1.0), (' of', 1.0), (' Victoria', 1.0), (',', 1.0), (' Australia', 1.0)]</t>
+          <t>[(' F', 1.0), ('awk', 1.0), ('ner', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' north', 1.0), (' of', 1.0), (' Melbourne', 1.0), (',', 1.0), (' Victoria', 1.0), (',', 1.0), (' Australia', 1.0)]</t>
         </is>
       </c>
       <c r="L92" t="n">
@@ -4896,7 +4870,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>What is the location of Fawkner?</t>
+          <t>What is the] loc^ation of `Fawkner?</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4909,12 +4883,12 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>What is the location of Fawkner? Answer: Fawkner is located in the state of Victoria, Australia. The city is located in the northern suburbs of Melbourne, the</t>
+          <t>What is the] loc^ation of `Fawkner? Answer: Fawkner is located in the north of Melbourne, Victoria, Australia. It is a suburb of Melbourne, Victoria, Australia</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Answer: Fawkner is located in the state of Victoria, Australia</t>
+          <t>Answer: Fawkner is located in the north of Melbourne, Victoria, Australia</t>
         </is>
       </c>
       <c r="G93" t="n">
@@ -4931,7 +4905,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>[(' F', 1.0), ('awk', 1.0), ('ner', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' state', 1.0), (' of', 1.0), (' Victoria', 1.0), (',', 1.0), (' Australia', 1.0)]</t>
+          <t>[(' F', 1.0), ('awk', 1.0), ('ner', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' north', 1.0), (' of', 1.0), (' Melbourne', 1.0), (',', 1.0), (' Victoria', 1.0), (',', 1.0), (' Australia', 1.0)]</t>
         </is>
       </c>
       <c r="L93" t="n">
@@ -4944,7 +4918,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>What is the location of Fawkner?</t>
+          <t>What is the] loc^ation of `Fawkner?</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4957,12 +4931,12 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>What is the location of Fawkner? Answer: Fawkner is located in the state of Victoria, Australia. The city is located in the northern suburbs of Melbourne, the</t>
+          <t>What is the] loc^ation of `Fawkner? Answer: Fawkner is located in the north of Melbourne, Victoria, Australia. It is a suburb of Melbourne, Victoria, Australia</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Answer: Fawkner is located in the state of Victoria, Australia</t>
+          <t>Answer: Fawkner is located in the north of Melbourne, Victoria, Australia</t>
         </is>
       </c>
       <c r="G94" t="n">
@@ -4979,7 +4953,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>[(' F', 1.0), ('awk', 1.0), ('ner', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' state', 1.0), (' of', 1.0), (' Victoria', 1.0), (',', 1.0), (' Australia', 1.0)]</t>
+          <t>[(' F', 1.0), ('awk', 1.0), ('ner', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' north', 1.0), (' of', 1.0), (' Melbourne', 1.0), (',', 1.0), (' Victoria', 1.0), (',', 1.0), (' Australia', 1.0)]</t>
         </is>
       </c>
       <c r="L94" t="n">
@@ -4992,7 +4966,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>What is the location of Fawkner?</t>
+          <t>What is the] loc^ation of `Fawkner?</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -5005,12 +4979,12 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>What is the location of Fawkner? Answer: Fawkner is located in the state of Victoria, Australia. The city is located in the northern suburbs of Melbourne, the</t>
+          <t>What is the] loc^ation of `Fawkner? Answer: Fawkner is located in the north of Melbourne, Victoria, Australia. It is a suburb of Melbourne, Victoria, Australia</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Answer: Fawkner is located in the state of Victoria, Australia</t>
+          <t>Answer: Fawkner is located in the north of Melbourne, Victoria, Australia</t>
         </is>
       </c>
       <c r="G95" t="n">
@@ -5027,7 +5001,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>[(' F', 1.0), ('awk', 1.0), ('ner', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' state', 1.0), (' of', 1.0), (' Victoria', 1.0), (',', 1.0), (' Australia', 1.0)]</t>
+          <t>[(' F', 1.0), ('awk', 1.0), ('ner', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' north', 1.0), (' of', 1.0), (' Melbourne', 1.0), (',', 1.0), (' Victoria', 1.0), (',', 1.0), (' Australia', 1.0)]</t>
         </is>
       </c>
       <c r="L95" t="n">
@@ -5040,7 +5014,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>What is the location of Fawkner?</t>
+          <t>What is the] loc^ation of `Fawkner?</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -5053,12 +5027,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>What is the location of Fawkner? Answer: Fawkner is located in the state of Victoria, Australia. The city is located in the northern suburbs of Melbourne, the</t>
+          <t>What is the] loc^ation of `Fawkner? Answer: Fawkner is located in the north of Melbourne, Victoria, Australia. It is a suburb of Melbourne. It is located</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Answer: Fawkner is located in the state of Victoria, Australia</t>
+          <t>Answer: Fawkner is located in the north of Melbourne, Victoria, Australia</t>
         </is>
       </c>
       <c r="G96" t="n">
@@ -5075,7 +5049,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>[(' F', 1.0), ('awk', 1.0), ('ner', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' state', 1.0), (' of', 1.0), (' Victoria', 1.0), (',', 1.0), (' Australia', 1.0)]</t>
+          <t>[(' F', 1.0), ('awk', 1.0), ('ner', 1.0), (' is', 1.0), (' located', 1.0), (' in', 1.0), (' the', 1.0), (' north', 1.0), (' of', 1.0), (' Melbourne', 1.0), (',', 1.0), (' Victoria', 1.0), (',', 1.0), (' Australia', 1.0)]</t>
         </is>
       </c>
       <c r="L96" t="n">
@@ -5088,7 +5062,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>What is the location of Abu Ghosh?</t>
+          <t>What$ is the location of$ Abu Gho+sh?</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -5101,7 +5075,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>What is the location of Abu Ghosh? Answer: Abu Ghosh is located in the Jerusalem District of Israel. It is located 10 km west of Jerusalem and 5 km</t>
+          <t>What$ is the location of$ Abu Gho+sh? Answer: Abu Ghosh is located in the Jerusalem District of Israel. It is located 10 km west of Jerusalem and 5 km</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -5136,7 +5110,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>What is the location of Abu Ghosh?</t>
+          <t>What$ is the location of$ Abu Gho+sh?</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -5149,7 +5123,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>What is the location of Abu Ghosh? Answer: Abu Ghosh is located in the Jerusalem District of Israel. The city is located 10 km west of Jerusalem and 5</t>
+          <t>What$ is the location of$ Abu Gho+sh? Answer: Abu Ghosh is located in the Jerusalem District of Israel. It is located 10 km west of Jerusalem and 5 km</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -5184,7 +5158,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>What is the location of Abu Ghosh?</t>
+          <t>What$ is the location of$ Abu Gho+sh?</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -5197,7 +5171,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>What is the location of Abu Ghosh? Answer: Abu Ghosh is located in the Jerusalem District of Israel. It is located 10 km west of Jerusalem and 5 km</t>
+          <t>What$ is the location of$ Abu Gho+sh? Answer: Abu Ghosh is located in the Jerusalem District of Israel. It is located 10 km west of Jerusalem and 5 km</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -5232,7 +5206,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>What is the location of Abu Ghosh?</t>
+          <t>What$ is the location of$ Abu Gho+sh?</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -5245,7 +5219,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>What is the location of Abu Ghosh? Answer: Abu Ghosh is located in the Jerusalem District of Israel. It is located 10 km west of Jerusalem and 5 km</t>
+          <t>What$ is the location of$ Abu Gho+sh? Answer: Abu Ghosh is located in the Jerusalem District of Israel. It is located 10 km west of Jerusalem and 5 km</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -5280,7 +5254,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>What is the location of Abu Ghosh?</t>
+          <t>What$ is the location of$ Abu Gho+sh?</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -5293,7 +5267,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>What is the location of Abu Ghosh? Answer: Abu Ghosh is located in the Jerusalem District of Israel. It is located 10 km west of Jerusalem and 5 km</t>
+          <t>What$ is the location of$ Abu Gho+sh? Answer: Abu Ghosh is located in the Jerusalem District of Israel. It is located 10 km west of Jerusalem and 5 km</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">

</xml_diff>